<commit_message>
Publish 20260506 REITs map site
</commit_message>
<xml_diff>
--- a/REITs_location_updating.xlsx
+++ b/REITs_location_updating.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\21076\Desktop\公募REITs地图项目\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{299F8A9E-2B24-44FD-8535-518BFDE3F739}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E3C398FA-7EAF-4E12-AD9A-5AAC70C714F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="648" uniqueCount="498">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="656" uniqueCount="504">
   <si>
     <t>证券代码</t>
   </si>
@@ -303,9 +303,6 @@
     <t>508017.SH</t>
   </si>
   <si>
-    <t>华夏金茂商业</t>
-  </si>
-  <si>
     <t>上海兴秀茂商业管理有限公司</t>
   </si>
   <si>
@@ -846,9 +843,6 @@
     <t>508091.SH</t>
   </si>
   <si>
-    <t>华夏凯德商业</t>
-  </si>
-  <si>
     <t>CAPITALAND MALL ASIA LIMITED,长沙凯亭咨询管理有限公司,广州凯云管理咨询有限公司,广州云凯商业管理有限公司</t>
   </si>
   <si>
@@ -1233,9 +1227,6 @@
     <t>180601.SZ</t>
   </si>
   <si>
-    <t>华夏华润商业</t>
-  </si>
-  <si>
     <t>华润商业资产控股有限公司</t>
   </si>
   <si>
@@ -1266,9 +1257,6 @@
     <t>180603.SZ</t>
   </si>
   <si>
-    <t>华夏大悦城商业</t>
-  </si>
-  <si>
     <t>卓远地产(成都)有限公司</t>
   </si>
   <si>
@@ -1299,9 +1287,6 @@
     <t>180606.SZ</t>
   </si>
   <si>
-    <t>中金中国绿发商业</t>
-  </si>
-  <si>
     <t>山东鲁能商业管理有限公司</t>
   </si>
   <si>
@@ -1312,9 +1297,6 @@
   </si>
   <si>
     <t>180607.SZ</t>
-  </si>
-  <si>
-    <t>华夏中海商业</t>
   </si>
   <si>
     <t>中海环宇商业发展(深圳)有限公司</t>
@@ -1525,6 +1507,48 @@
   </si>
   <si>
     <t>{钱江通道及接线工程钱江隧道段}|{钱江通道及接线工程钱江隧道段}</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>中航北京昌保租赁住房</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>华夏金茂消费</t>
+  </si>
+  <si>
+    <t>华夏凯德消费</t>
+  </si>
+  <si>
+    <t>华夏华润消费</t>
+  </si>
+  <si>
+    <t>华夏大悦城消费</t>
+  </si>
+  <si>
+    <t>中金中国绿发消费</t>
+  </si>
+  <si>
+    <t>华夏中海消费</t>
+  </si>
+  <si>
+    <t>北京市</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>{滟澜新宸项目，国瑞熙院项目，未来融尚家园项目}</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>180503.SZ</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>北京昌鑫建设投资有限公司</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>滟澜新宸项目，国瑞熙院项目，未来融尚家园项目</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
@@ -1793,7 +1817,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H81"/>
+  <dimension ref="A1:H82"/>
   <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10.54296875" customWidth="1"/>
@@ -1853,7 +1877,7 @@
         <v>13</v>
       </c>
       <c r="H2" t="s">
-        <v>456</v>
+        <v>450</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
@@ -1879,7 +1903,7 @@
         <v>20</v>
       </c>
       <c r="H3" t="s">
-        <v>457</v>
+        <v>451</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
@@ -1931,7 +1955,7 @@
         <v>31</v>
       </c>
       <c r="H5" t="s">
-        <v>458</v>
+        <v>452</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
@@ -1983,7 +2007,7 @@
         <v>45</v>
       </c>
       <c r="H7" t="s">
-        <v>459</v>
+        <v>453</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
@@ -2087,7 +2111,7 @@
         <v>57</v>
       </c>
       <c r="H11" t="s">
-        <v>460</v>
+        <v>454</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.25">
@@ -2113,7 +2137,7 @@
         <v>31</v>
       </c>
       <c r="H12" t="s">
-        <v>461</v>
+        <v>455</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
@@ -2139,7 +2163,7 @@
         <v>13</v>
       </c>
       <c r="H13" t="s">
-        <v>462</v>
+        <v>456</v>
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.25">
@@ -2199,91 +2223,91 @@
         <v>91</v>
       </c>
       <c r="B16" t="s">
+        <v>493</v>
+      </c>
+      <c r="C16" t="s">
         <v>92</v>
       </c>
-      <c r="C16" t="s">
+      <c r="D16" t="s">
         <v>93</v>
-      </c>
-      <c r="D16" t="s">
-        <v>94</v>
       </c>
       <c r="E16" t="s">
         <v>25</v>
       </c>
       <c r="F16" t="s">
+        <v>94</v>
+      </c>
+      <c r="G16" t="s">
         <v>95</v>
       </c>
-      <c r="G16" t="s">
+      <c r="H16" t="s">
         <v>96</v>
-      </c>
-      <c r="H16" t="s">
-        <v>97</v>
       </c>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
+        <v>97</v>
+      </c>
+      <c r="B17" t="s">
         <v>98</v>
       </c>
-      <c r="B17" t="s">
+      <c r="C17" t="s">
         <v>99</v>
       </c>
-      <c r="C17" t="s">
+      <c r="D17" t="s">
         <v>100</v>
-      </c>
-      <c r="D17" t="s">
-        <v>101</v>
       </c>
       <c r="E17" t="s">
         <v>18</v>
       </c>
       <c r="F17" t="s">
+        <v>101</v>
+      </c>
+      <c r="G17" t="s">
         <v>102</v>
       </c>
-      <c r="G17" t="s">
+      <c r="H17" t="s">
         <v>103</v>
-      </c>
-      <c r="H17" t="s">
-        <v>104</v>
       </c>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
+        <v>104</v>
+      </c>
+      <c r="B18" t="s">
         <v>105</v>
       </c>
-      <c r="B18" t="s">
+      <c r="C18" t="s">
         <v>106</v>
       </c>
-      <c r="C18" t="s">
+      <c r="D18" t="s">
         <v>107</v>
-      </c>
-      <c r="D18" t="s">
-        <v>108</v>
       </c>
       <c r="E18" t="s">
         <v>12</v>
       </c>
       <c r="F18" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="G18" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="H18" t="s">
-        <v>463</v>
+        <v>457</v>
       </c>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
+        <v>109</v>
+      </c>
+      <c r="B19" t="s">
         <v>110</v>
       </c>
-      <c r="B19" t="s">
+      <c r="C19" t="s">
         <v>111</v>
       </c>
-      <c r="C19" t="s">
+      <c r="D19" t="s">
         <v>112</v>
-      </c>
-      <c r="D19" t="s">
-        <v>113</v>
       </c>
       <c r="E19" t="s">
         <v>12</v>
@@ -2295,154 +2319,154 @@
         <v>13</v>
       </c>
       <c r="H19" t="s">
-        <v>464</v>
+        <v>458</v>
       </c>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
+        <v>113</v>
+      </c>
+      <c r="B20" t="s">
         <v>114</v>
       </c>
-      <c r="B20" t="s">
+      <c r="C20" t="s">
         <v>115</v>
       </c>
-      <c r="C20" t="s">
+      <c r="D20" t="s">
         <v>116</v>
-      </c>
-      <c r="D20" t="s">
-        <v>117</v>
       </c>
       <c r="E20" t="s">
         <v>12</v>
       </c>
       <c r="F20" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="G20" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="H20" t="s">
-        <v>465</v>
+        <v>459</v>
       </c>
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
+        <v>118</v>
+      </c>
+      <c r="B21" t="s">
         <v>119</v>
       </c>
-      <c r="B21" t="s">
+      <c r="C21" t="s">
         <v>120</v>
       </c>
-      <c r="C21" t="s">
+      <c r="D21" t="s">
         <v>121</v>
-      </c>
-      <c r="D21" t="s">
-        <v>122</v>
       </c>
       <c r="E21" t="s">
         <v>82</v>
       </c>
       <c r="F21" t="s">
+        <v>122</v>
+      </c>
+      <c r="G21" t="s">
         <v>123</v>
       </c>
-      <c r="G21" t="s">
+      <c r="H21" t="s">
         <v>124</v>
-      </c>
-      <c r="H21" t="s">
-        <v>125</v>
       </c>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
+        <v>125</v>
+      </c>
+      <c r="B22" t="s">
         <v>126</v>
       </c>
-      <c r="B22" t="s">
+      <c r="C22" t="s">
         <v>127</v>
       </c>
-      <c r="C22" t="s">
+      <c r="D22" t="s">
         <v>128</v>
-      </c>
-      <c r="D22" t="s">
-        <v>129</v>
       </c>
       <c r="E22" t="s">
         <v>12</v>
       </c>
       <c r="F22" t="s">
+        <v>129</v>
+      </c>
+      <c r="G22" t="s">
         <v>130</v>
       </c>
-      <c r="G22" t="s">
-        <v>131</v>
-      </c>
       <c r="H22" t="s">
-        <v>466</v>
+        <v>460</v>
       </c>
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
+        <v>131</v>
+      </c>
+      <c r="B23" t="s">
         <v>132</v>
       </c>
-      <c r="B23" t="s">
+      <c r="C23" t="s">
         <v>133</v>
       </c>
-      <c r="C23" t="s">
+      <c r="D23" t="s">
         <v>134</v>
-      </c>
-      <c r="D23" t="s">
-        <v>135</v>
       </c>
       <c r="E23" t="s">
         <v>82</v>
       </c>
       <c r="F23" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="G23" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="H23" t="s">
-        <v>467</v>
+        <v>461</v>
       </c>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
+        <v>136</v>
+      </c>
+      <c r="B24" t="s">
         <v>137</v>
       </c>
-      <c r="B24" t="s">
+      <c r="C24" t="s">
         <v>138</v>
       </c>
-      <c r="C24" t="s">
+      <c r="D24" t="s">
         <v>139</v>
-      </c>
-      <c r="D24" t="s">
-        <v>140</v>
       </c>
       <c r="E24" t="s">
         <v>12</v>
       </c>
       <c r="F24" t="s">
+        <v>140</v>
+      </c>
+      <c r="G24" t="s">
         <v>141</v>
       </c>
-      <c r="G24" t="s">
-        <v>142</v>
-      </c>
       <c r="H24" t="s">
-        <v>468</v>
+        <v>462</v>
       </c>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
+        <v>142</v>
+      </c>
+      <c r="B25" t="s">
         <v>143</v>
       </c>
-      <c r="B25" t="s">
+      <c r="C25" t="s">
         <v>144</v>
       </c>
-      <c r="C25" t="s">
+      <c r="D25" t="s">
         <v>145</v>
       </c>
-      <c r="D25" t="s">
+      <c r="E25" t="s">
         <v>146</v>
-      </c>
-      <c r="E25" t="s">
-        <v>147</v>
       </c>
       <c r="F25" t="s">
         <v>13</v>
@@ -2451,73 +2475,73 @@
         <v>13</v>
       </c>
       <c r="H25" t="s">
-        <v>469</v>
+        <v>463</v>
       </c>
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
+        <v>147</v>
+      </c>
+      <c r="B26" t="s">
         <v>148</v>
       </c>
-      <c r="B26" t="s">
+      <c r="C26" t="s">
         <v>149</v>
       </c>
-      <c r="C26" t="s">
+      <c r="D26" t="s">
         <v>150</v>
-      </c>
-      <c r="D26" t="s">
-        <v>151</v>
       </c>
       <c r="E26" t="s">
         <v>18</v>
       </c>
       <c r="F26" t="s">
+        <v>151</v>
+      </c>
+      <c r="G26" t="s">
         <v>152</v>
       </c>
-      <c r="G26" t="s">
+      <c r="H26" t="s">
         <v>153</v>
-      </c>
-      <c r="H26" t="s">
-        <v>154</v>
       </c>
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
+        <v>154</v>
+      </c>
+      <c r="B27" t="s">
         <v>155</v>
       </c>
-      <c r="B27" t="s">
+      <c r="C27" t="s">
         <v>156</v>
       </c>
-      <c r="C27" t="s">
+      <c r="D27" t="s">
         <v>157</v>
-      </c>
-      <c r="D27" t="s">
-        <v>158</v>
       </c>
       <c r="E27" t="s">
         <v>18</v>
       </c>
       <c r="F27" t="s">
+        <v>158</v>
+      </c>
+      <c r="G27" t="s">
         <v>159</v>
       </c>
-      <c r="G27" t="s">
+      <c r="H27" t="s">
         <v>160</v>
-      </c>
-      <c r="H27" t="s">
-        <v>161</v>
       </c>
     </row>
     <row r="28" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
+        <v>161</v>
+      </c>
+      <c r="B28" t="s">
         <v>162</v>
       </c>
-      <c r="B28" t="s">
+      <c r="C28" t="s">
         <v>163</v>
       </c>
-      <c r="C28" t="s">
+      <c r="D28" t="s">
         <v>164</v>
-      </c>
-      <c r="D28" t="s">
-        <v>165</v>
       </c>
       <c r="E28" t="s">
         <v>12</v>
@@ -2529,24 +2553,24 @@
         <v>31</v>
       </c>
       <c r="H28" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
     </row>
     <row r="29" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
+        <v>166</v>
+      </c>
+      <c r="B29" t="s">
         <v>167</v>
       </c>
-      <c r="B29" t="s">
+      <c r="C29" t="s">
         <v>168</v>
       </c>
-      <c r="C29" t="s">
+      <c r="D29" t="s">
         <v>169</v>
       </c>
-      <c r="D29" t="s">
+      <c r="E29" t="s">
         <v>170</v>
-      </c>
-      <c r="E29" t="s">
-        <v>171</v>
       </c>
       <c r="F29" t="s">
         <v>13</v>
@@ -2555,24 +2579,24 @@
         <v>13</v>
       </c>
       <c r="H29" t="s">
-        <v>470</v>
+        <v>464</v>
       </c>
     </row>
     <row r="30" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
+        <v>171</v>
+      </c>
+      <c r="B30" t="s">
         <v>172</v>
       </c>
-      <c r="B30" t="s">
+      <c r="C30" t="s">
         <v>173</v>
       </c>
-      <c r="C30" t="s">
+      <c r="D30" t="s">
         <v>174</v>
       </c>
-      <c r="D30" t="s">
-        <v>175</v>
-      </c>
       <c r="E30" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="F30" t="s">
         <v>13</v>
@@ -2581,128 +2605,128 @@
         <v>13</v>
       </c>
       <c r="H30" t="s">
-        <v>471</v>
+        <v>465</v>
       </c>
     </row>
     <row r="31" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
+        <v>175</v>
+      </c>
+      <c r="B31" t="s">
         <v>176</v>
       </c>
-      <c r="B31" t="s">
+      <c r="C31" t="s">
         <v>177</v>
       </c>
-      <c r="C31" t="s">
+      <c r="D31" t="s">
         <v>178</v>
       </c>
-      <c r="D31" t="s">
+      <c r="E31" t="s">
+        <v>170</v>
+      </c>
+      <c r="F31" t="s">
         <v>179</v>
       </c>
-      <c r="E31" t="s">
-        <v>171</v>
-      </c>
-      <c r="F31" t="s">
+      <c r="G31" t="s">
         <v>180</v>
       </c>
-      <c r="G31" t="s">
-        <v>181</v>
-      </c>
       <c r="H31" t="s">
-        <v>472</v>
+        <v>466</v>
       </c>
     </row>
     <row r="32" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
+        <v>181</v>
+      </c>
+      <c r="B32" t="s">
         <v>182</v>
       </c>
-      <c r="B32" t="s">
+      <c r="C32" t="s">
         <v>183</v>
       </c>
-      <c r="C32" t="s">
+      <c r="D32" t="s">
         <v>184</v>
       </c>
-      <c r="D32" t="s">
+      <c r="E32" t="s">
+        <v>146</v>
+      </c>
+      <c r="F32" t="s">
         <v>185</v>
       </c>
-      <c r="E32" t="s">
-        <v>147</v>
-      </c>
-      <c r="F32" t="s">
+      <c r="G32" t="s">
         <v>186</v>
       </c>
-      <c r="G32" t="s">
-        <v>187</v>
-      </c>
       <c r="H32" t="s">
-        <v>473</v>
+        <v>467</v>
       </c>
     </row>
     <row r="33" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
+        <v>187</v>
+      </c>
+      <c r="B33" t="s">
         <v>188</v>
       </c>
-      <c r="B33" t="s">
+      <c r="C33" t="s">
         <v>189</v>
       </c>
-      <c r="C33" t="s">
+      <c r="D33" t="s">
         <v>190</v>
       </c>
-      <c r="D33" t="s">
+      <c r="E33" t="s">
         <v>191</v>
       </c>
-      <c r="E33" t="s">
+      <c r="F33" t="s">
+        <v>129</v>
+      </c>
+      <c r="G33" t="s">
+        <v>130</v>
+      </c>
+      <c r="H33" t="s">
         <v>192</v>
-      </c>
-      <c r="F33" t="s">
-        <v>130</v>
-      </c>
-      <c r="G33" t="s">
-        <v>131</v>
-      </c>
-      <c r="H33" t="s">
-        <v>193</v>
       </c>
     </row>
     <row r="34" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
+        <v>193</v>
+      </c>
+      <c r="B34" t="s">
         <v>194</v>
       </c>
-      <c r="B34" t="s">
+      <c r="C34" t="s">
         <v>195</v>
       </c>
-      <c r="C34" t="s">
+      <c r="D34" t="s">
         <v>196</v>
-      </c>
-      <c r="D34" t="s">
-        <v>197</v>
       </c>
       <c r="E34" t="s">
         <v>18</v>
       </c>
       <c r="F34" t="s">
+        <v>129</v>
+      </c>
+      <c r="G34" t="s">
         <v>130</v>
       </c>
-      <c r="G34" t="s">
-        <v>131</v>
-      </c>
       <c r="H34" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
     </row>
     <row r="35" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
+        <v>198</v>
+      </c>
+      <c r="B35" t="s">
         <v>199</v>
       </c>
-      <c r="B35" t="s">
+      <c r="C35" t="s">
         <v>200</v>
       </c>
-      <c r="C35" t="s">
+      <c r="D35" t="s">
         <v>201</v>
       </c>
-      <c r="D35" t="s">
-        <v>202</v>
-      </c>
       <c r="E35" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="F35" t="s">
         <v>31</v>
@@ -2711,50 +2735,50 @@
         <v>31</v>
       </c>
       <c r="H35" t="s">
-        <v>474</v>
+        <v>468</v>
       </c>
     </row>
     <row r="36" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
+        <v>202</v>
+      </c>
+      <c r="B36" t="s">
         <v>203</v>
       </c>
-      <c r="B36" t="s">
+      <c r="C36" t="s">
         <v>204</v>
       </c>
-      <c r="C36" t="s">
+      <c r="D36" t="s">
         <v>205</v>
-      </c>
-      <c r="D36" t="s">
-        <v>206</v>
       </c>
       <c r="E36" t="s">
         <v>18</v>
       </c>
       <c r="F36" t="s">
+        <v>206</v>
+      </c>
+      <c r="G36" t="s">
+        <v>130</v>
+      </c>
+      <c r="H36" t="s">
         <v>207</v>
-      </c>
-      <c r="G36" t="s">
-        <v>131</v>
-      </c>
-      <c r="H36" t="s">
-        <v>208</v>
       </c>
     </row>
     <row r="37" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
+        <v>208</v>
+      </c>
+      <c r="B37" t="s">
         <v>209</v>
       </c>
-      <c r="B37" t="s">
+      <c r="C37" t="s">
         <v>210</v>
       </c>
-      <c r="C37" t="s">
+      <c r="D37" t="s">
         <v>211</v>
       </c>
-      <c r="D37" t="s">
-        <v>212</v>
-      </c>
       <c r="E37" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="F37" t="s">
         <v>13</v>
@@ -2763,47 +2787,47 @@
         <v>13</v>
       </c>
       <c r="H37" t="s">
-        <v>475</v>
+        <v>469</v>
       </c>
     </row>
     <row r="38" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
+        <v>212</v>
+      </c>
+      <c r="B38" t="s">
         <v>213</v>
       </c>
-      <c r="B38" t="s">
+      <c r="C38" t="s">
         <v>214</v>
       </c>
-      <c r="C38" t="s">
+      <c r="D38" t="s">
         <v>215</v>
       </c>
-      <c r="D38" t="s">
+      <c r="E38" t="s">
+        <v>170</v>
+      </c>
+      <c r="F38" t="s">
+        <v>129</v>
+      </c>
+      <c r="G38" t="s">
+        <v>130</v>
+      </c>
+      <c r="H38" t="s">
         <v>216</v>
-      </c>
-      <c r="E38" t="s">
-        <v>171</v>
-      </c>
-      <c r="F38" t="s">
-        <v>130</v>
-      </c>
-      <c r="G38" t="s">
-        <v>131</v>
-      </c>
-      <c r="H38" t="s">
-        <v>217</v>
       </c>
     </row>
     <row r="39" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
+        <v>217</v>
+      </c>
+      <c r="B39" t="s">
         <v>218</v>
       </c>
-      <c r="B39" t="s">
+      <c r="C39" t="s">
         <v>219</v>
       </c>
-      <c r="C39" t="s">
+      <c r="D39" t="s">
         <v>220</v>
-      </c>
-      <c r="D39" t="s">
-        <v>221</v>
       </c>
       <c r="E39" t="s">
         <v>12</v>
@@ -2815,255 +2839,255 @@
         <v>31</v>
       </c>
       <c r="H39" t="s">
-        <v>476</v>
+        <v>470</v>
       </c>
     </row>
     <row r="40" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
+        <v>221</v>
+      </c>
+      <c r="B40" t="s">
         <v>222</v>
       </c>
-      <c r="B40" t="s">
+      <c r="C40" t="s">
         <v>223</v>
       </c>
-      <c r="C40" t="s">
+      <c r="D40" t="s">
         <v>224</v>
-      </c>
-      <c r="D40" t="s">
-        <v>225</v>
       </c>
       <c r="E40" t="s">
         <v>25</v>
       </c>
       <c r="F40" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="G40" t="s">
         <v>20</v>
       </c>
       <c r="H40" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
     </row>
     <row r="41" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
+        <v>227</v>
+      </c>
+      <c r="B41" t="s">
         <v>228</v>
       </c>
-      <c r="B41" t="s">
+      <c r="C41" t="s">
         <v>229</v>
       </c>
-      <c r="C41" t="s">
+      <c r="D41" t="s">
         <v>230</v>
       </c>
-      <c r="D41" t="s">
+      <c r="E41" t="s">
+        <v>170</v>
+      </c>
+      <c r="F41" t="s">
+        <v>108</v>
+      </c>
+      <c r="G41" t="s">
+        <v>102</v>
+      </c>
+      <c r="H41" t="s">
         <v>231</v>
-      </c>
-      <c r="E41" t="s">
-        <v>171</v>
-      </c>
-      <c r="F41" t="s">
-        <v>109</v>
-      </c>
-      <c r="G41" t="s">
-        <v>103</v>
-      </c>
-      <c r="H41" t="s">
-        <v>232</v>
       </c>
     </row>
     <row r="42" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
+        <v>232</v>
+      </c>
+      <c r="B42" t="s">
         <v>233</v>
       </c>
-      <c r="B42" t="s">
+      <c r="C42" t="s">
         <v>234</v>
       </c>
-      <c r="C42" t="s">
+      <c r="D42" t="s">
         <v>235</v>
       </c>
-      <c r="D42" t="s">
+      <c r="E42" t="s">
+        <v>146</v>
+      </c>
+      <c r="F42" t="s">
+        <v>129</v>
+      </c>
+      <c r="G42" t="s">
+        <v>130</v>
+      </c>
+      <c r="H42" t="s">
         <v>236</v>
-      </c>
-      <c r="E42" t="s">
-        <v>147</v>
-      </c>
-      <c r="F42" t="s">
-        <v>130</v>
-      </c>
-      <c r="G42" t="s">
-        <v>131</v>
-      </c>
-      <c r="H42" t="s">
-        <v>237</v>
       </c>
     </row>
     <row r="43" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
+        <v>237</v>
+      </c>
+      <c r="B43" t="s">
         <v>238</v>
       </c>
-      <c r="B43" t="s">
+      <c r="C43" t="s">
         <v>239</v>
       </c>
-      <c r="C43" t="s">
+      <c r="D43" t="s">
         <v>240</v>
-      </c>
-      <c r="D43" t="s">
-        <v>241</v>
       </c>
       <c r="E43" t="s">
         <v>18</v>
       </c>
       <c r="F43" t="s">
+        <v>241</v>
+      </c>
+      <c r="G43" t="s">
         <v>242</v>
       </c>
-      <c r="G43" t="s">
+      <c r="H43" t="s">
         <v>243</v>
-      </c>
-      <c r="H43" t="s">
-        <v>244</v>
       </c>
     </row>
     <row r="44" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
+        <v>244</v>
+      </c>
+      <c r="B44" t="s">
         <v>245</v>
       </c>
-      <c r="B44" t="s">
+      <c r="C44" t="s">
         <v>246</v>
       </c>
-      <c r="C44" t="s">
+      <c r="D44" t="s">
         <v>247</v>
       </c>
-      <c r="D44" t="s">
+      <c r="E44" t="s">
         <v>248</v>
       </c>
-      <c r="E44" t="s">
+      <c r="F44" t="s">
         <v>249</v>
-      </c>
-      <c r="F44" t="s">
-        <v>250</v>
       </c>
       <c r="G44" t="s">
         <v>51</v>
       </c>
       <c r="H44" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
     </row>
     <row r="45" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
+        <v>251</v>
+      </c>
+      <c r="B45" t="s">
         <v>252</v>
       </c>
-      <c r="B45" t="s">
+      <c r="C45" t="s">
         <v>253</v>
       </c>
-      <c r="C45" t="s">
+      <c r="D45" t="s">
         <v>254</v>
-      </c>
-      <c r="D45" t="s">
-        <v>255</v>
       </c>
       <c r="E45" t="s">
         <v>12</v>
       </c>
       <c r="F45" t="s">
+        <v>255</v>
+      </c>
+      <c r="G45" t="s">
         <v>256</v>
       </c>
-      <c r="G45" t="s">
+      <c r="H45" t="s">
         <v>257</v>
-      </c>
-      <c r="H45" t="s">
-        <v>258</v>
       </c>
     </row>
     <row r="46" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
+        <v>258</v>
+      </c>
+      <c r="B46" t="s">
         <v>259</v>
       </c>
-      <c r="B46" t="s">
+      <c r="C46" t="s">
         <v>260</v>
       </c>
-      <c r="C46" t="s">
+      <c r="D46" t="s">
         <v>261</v>
-      </c>
-      <c r="D46" t="s">
-        <v>262</v>
       </c>
       <c r="E46" t="s">
         <v>82</v>
       </c>
       <c r="F46" t="s">
+        <v>262</v>
+      </c>
+      <c r="G46" t="s">
         <v>263</v>
       </c>
-      <c r="G46" t="s">
+      <c r="H46" t="s">
         <v>264</v>
-      </c>
-      <c r="H46" t="s">
-        <v>265</v>
       </c>
     </row>
     <row r="47" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
+        <v>265</v>
+      </c>
+      <c r="B47" t="s">
         <v>266</v>
       </c>
-      <c r="B47" t="s">
+      <c r="C47" t="s">
         <v>267</v>
       </c>
-      <c r="C47" t="s">
+      <c r="D47" t="s">
         <v>268</v>
       </c>
-      <c r="D47" t="s">
+      <c r="E47" t="s">
+        <v>170</v>
+      </c>
+      <c r="F47" t="s">
         <v>269</v>
       </c>
-      <c r="E47" t="s">
-        <v>171</v>
-      </c>
-      <c r="F47" t="s">
+      <c r="G47" t="s">
         <v>270</v>
       </c>
-      <c r="G47" t="s">
-        <v>271</v>
-      </c>
       <c r="H47" t="s">
-        <v>477</v>
+        <v>471</v>
       </c>
     </row>
     <row r="48" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
+        <v>271</v>
+      </c>
+      <c r="B48" t="s">
+        <v>494</v>
+      </c>
+      <c r="C48" t="s">
         <v>272</v>
       </c>
-      <c r="B48" t="s">
+      <c r="D48" t="s">
         <v>273</v>
-      </c>
-      <c r="C48" t="s">
-        <v>274</v>
-      </c>
-      <c r="D48" t="s">
-        <v>275</v>
       </c>
       <c r="E48" t="s">
         <v>25</v>
       </c>
       <c r="F48" t="s">
+        <v>274</v>
+      </c>
+      <c r="G48" t="s">
+        <v>275</v>
+      </c>
+      <c r="H48" t="s">
         <v>276</v>
-      </c>
-      <c r="G48" t="s">
-        <v>277</v>
-      </c>
-      <c r="H48" t="s">
-        <v>278</v>
       </c>
     </row>
     <row r="49" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
+        <v>277</v>
+      </c>
+      <c r="B49" t="s">
+        <v>278</v>
+      </c>
+      <c r="C49" t="s">
         <v>279</v>
       </c>
-      <c r="B49" t="s">
+      <c r="D49" t="s">
         <v>280</v>
-      </c>
-      <c r="C49" t="s">
-        <v>281</v>
-      </c>
-      <c r="D49" t="s">
-        <v>282</v>
       </c>
       <c r="E49" t="s">
         <v>12</v>
@@ -3075,99 +3099,99 @@
         <v>31</v>
       </c>
       <c r="H49" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
     </row>
     <row r="50" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
+        <v>282</v>
+      </c>
+      <c r="B50" t="s">
+        <v>283</v>
+      </c>
+      <c r="C50" t="s">
         <v>284</v>
       </c>
-      <c r="B50" t="s">
+      <c r="D50" t="s">
         <v>285</v>
-      </c>
-      <c r="C50" t="s">
-        <v>286</v>
-      </c>
-      <c r="D50" t="s">
-        <v>287</v>
       </c>
       <c r="E50" t="s">
         <v>82</v>
       </c>
       <c r="F50" t="s">
-        <v>288</v>
+        <v>286</v>
       </c>
       <c r="G50" t="s">
-        <v>289</v>
+        <v>287</v>
       </c>
       <c r="H50" t="s">
-        <v>478</v>
+        <v>472</v>
       </c>
     </row>
     <row r="51" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
+        <v>288</v>
+      </c>
+      <c r="B51" t="s">
+        <v>289</v>
+      </c>
+      <c r="C51" t="s">
         <v>290</v>
       </c>
-      <c r="B51" t="s">
+      <c r="D51" t="s">
         <v>291</v>
-      </c>
-      <c r="C51" t="s">
-        <v>292</v>
-      </c>
-      <c r="D51" t="s">
-        <v>293</v>
       </c>
       <c r="E51" t="s">
         <v>12</v>
       </c>
       <c r="F51" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="G51" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="H51" t="s">
-        <v>294</v>
+        <v>292</v>
       </c>
     </row>
     <row r="52" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
+        <v>293</v>
+      </c>
+      <c r="B52" t="s">
+        <v>294</v>
+      </c>
+      <c r="C52" t="s">
         <v>295</v>
       </c>
-      <c r="B52" t="s">
+      <c r="D52" t="s">
         <v>296</v>
       </c>
-      <c r="C52" t="s">
+      <c r="E52" t="s">
+        <v>170</v>
+      </c>
+      <c r="F52" t="s">
         <v>297</v>
       </c>
-      <c r="D52" t="s">
+      <c r="G52" t="s">
         <v>298</v>
       </c>
-      <c r="E52" t="s">
-        <v>171</v>
-      </c>
-      <c r="F52" t="s">
+      <c r="H52" t="s">
         <v>299</v>
-      </c>
-      <c r="G52" t="s">
-        <v>300</v>
-      </c>
-      <c r="H52" t="s">
-        <v>301</v>
       </c>
     </row>
     <row r="53" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
+        <v>300</v>
+      </c>
+      <c r="B53" t="s">
+        <v>301</v>
+      </c>
+      <c r="C53" t="s">
         <v>302</v>
       </c>
-      <c r="B53" t="s">
+      <c r="D53" t="s">
         <v>303</v>
-      </c>
-      <c r="C53" t="s">
-        <v>304</v>
-      </c>
-      <c r="D53" t="s">
-        <v>305</v>
       </c>
       <c r="E53" t="s">
         <v>12</v>
@@ -3179,73 +3203,73 @@
         <v>31</v>
       </c>
       <c r="H53" t="s">
-        <v>479</v>
+        <v>473</v>
       </c>
     </row>
     <row r="54" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
+        <v>304</v>
+      </c>
+      <c r="B54" t="s">
+        <v>305</v>
+      </c>
+      <c r="C54" t="s">
         <v>306</v>
       </c>
-      <c r="B54" t="s">
+      <c r="D54" t="s">
         <v>307</v>
-      </c>
-      <c r="C54" t="s">
-        <v>308</v>
-      </c>
-      <c r="D54" t="s">
-        <v>309</v>
       </c>
       <c r="E54" t="s">
         <v>12</v>
       </c>
       <c r="F54" t="s">
-        <v>310</v>
+        <v>308</v>
       </c>
       <c r="G54" t="s">
-        <v>311</v>
+        <v>309</v>
       </c>
       <c r="H54" t="s">
-        <v>480</v>
+        <v>474</v>
       </c>
     </row>
     <row r="55" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
+        <v>310</v>
+      </c>
+      <c r="B55" t="s">
+        <v>311</v>
+      </c>
+      <c r="C55" t="s">
         <v>312</v>
       </c>
-      <c r="B55" t="s">
+      <c r="D55" t="s">
         <v>313</v>
-      </c>
-      <c r="C55" t="s">
-        <v>314</v>
-      </c>
-      <c r="D55" t="s">
-        <v>315</v>
       </c>
       <c r="E55" t="s">
         <v>12</v>
       </c>
       <c r="F55" t="s">
+        <v>314</v>
+      </c>
+      <c r="G55" t="s">
+        <v>315</v>
+      </c>
+      <c r="H55" t="s">
         <v>316</v>
-      </c>
-      <c r="G55" t="s">
-        <v>317</v>
-      </c>
-      <c r="H55" t="s">
-        <v>318</v>
       </c>
     </row>
     <row r="56" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
+        <v>317</v>
+      </c>
+      <c r="B56" t="s">
+        <v>318</v>
+      </c>
+      <c r="C56" t="s">
         <v>319</v>
       </c>
-      <c r="B56" t="s">
-        <v>320</v>
-      </c>
-      <c r="C56" t="s">
-        <v>321</v>
-      </c>
       <c r="D56" s="2" t="s">
-        <v>492</v>
+        <v>486</v>
       </c>
       <c r="E56" t="s">
         <v>12</v>
@@ -3257,411 +3281,411 @@
         <v>20</v>
       </c>
       <c r="H56" t="s">
-        <v>481</v>
+        <v>475</v>
       </c>
     </row>
     <row r="57" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
+        <v>320</v>
+      </c>
+      <c r="B57" t="s">
+        <v>321</v>
+      </c>
+      <c r="C57" t="s">
         <v>322</v>
       </c>
-      <c r="B57" t="s">
+      <c r="D57" t="s">
         <v>323</v>
-      </c>
-      <c r="C57" t="s">
-        <v>324</v>
-      </c>
-      <c r="D57" t="s">
-        <v>325</v>
       </c>
       <c r="E57" t="s">
         <v>12</v>
       </c>
       <c r="F57" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
       <c r="G57" t="s">
-        <v>311</v>
+        <v>309</v>
       </c>
       <c r="H57" t="s">
-        <v>482</v>
+        <v>476</v>
       </c>
     </row>
     <row r="58" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
+        <v>325</v>
+      </c>
+      <c r="B58" t="s">
+        <v>326</v>
+      </c>
+      <c r="C58" t="s">
         <v>327</v>
       </c>
-      <c r="B58" t="s">
+      <c r="D58" t="s">
         <v>328</v>
-      </c>
-      <c r="C58" t="s">
-        <v>329</v>
-      </c>
-      <c r="D58" t="s">
-        <v>330</v>
       </c>
       <c r="E58" t="s">
         <v>12</v>
       </c>
       <c r="F58" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
       <c r="G58" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="H58" t="s">
-        <v>483</v>
+        <v>477</v>
       </c>
     </row>
     <row r="59" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
+        <v>330</v>
+      </c>
+      <c r="B59" t="s">
+        <v>331</v>
+      </c>
+      <c r="C59" t="s">
         <v>332</v>
       </c>
-      <c r="B59" t="s">
+      <c r="D59" t="s">
         <v>333</v>
-      </c>
-      <c r="C59" t="s">
-        <v>334</v>
-      </c>
-      <c r="D59" t="s">
-        <v>335</v>
       </c>
       <c r="E59" t="s">
         <v>18</v>
       </c>
       <c r="F59" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
       <c r="G59" t="s">
-        <v>311</v>
+        <v>309</v>
       </c>
       <c r="H59" t="s">
-        <v>336</v>
+        <v>334</v>
       </c>
     </row>
     <row r="60" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
+        <v>335</v>
+      </c>
+      <c r="B60" t="s">
+        <v>336</v>
+      </c>
+      <c r="C60" t="s">
         <v>337</v>
       </c>
-      <c r="B60" t="s">
+      <c r="D60" t="s">
         <v>338</v>
-      </c>
-      <c r="C60" t="s">
-        <v>339</v>
-      </c>
-      <c r="D60" t="s">
-        <v>340</v>
       </c>
       <c r="E60" t="s">
         <v>18</v>
       </c>
       <c r="F60" t="s">
+        <v>339</v>
+      </c>
+      <c r="G60" t="s">
+        <v>340</v>
+      </c>
+      <c r="H60" t="s">
         <v>341</v>
-      </c>
-      <c r="G60" t="s">
-        <v>342</v>
-      </c>
-      <c r="H60" t="s">
-        <v>343</v>
       </c>
     </row>
     <row r="61" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
+        <v>342</v>
+      </c>
+      <c r="B61" t="s">
+        <v>343</v>
+      </c>
+      <c r="C61" t="s">
         <v>344</v>
       </c>
-      <c r="B61" t="s">
+      <c r="D61" t="s">
         <v>345</v>
-      </c>
-      <c r="C61" t="s">
-        <v>346</v>
-      </c>
-      <c r="D61" t="s">
-        <v>347</v>
       </c>
       <c r="E61" t="s">
         <v>18</v>
       </c>
       <c r="F61" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
       <c r="G61" t="s">
         <v>64</v>
       </c>
       <c r="H61" t="s">
-        <v>349</v>
+        <v>347</v>
       </c>
     </row>
     <row r="62" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
+        <v>348</v>
+      </c>
+      <c r="B62" t="s">
+        <v>349</v>
+      </c>
+      <c r="C62" t="s">
         <v>350</v>
       </c>
-      <c r="B62" t="s">
+      <c r="D62" t="s">
         <v>351</v>
       </c>
-      <c r="C62" t="s">
-        <v>352</v>
-      </c>
-      <c r="D62" t="s">
-        <v>353</v>
-      </c>
       <c r="E62" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="F62" t="s">
-        <v>310</v>
+        <v>308</v>
       </c>
       <c r="G62" t="s">
-        <v>311</v>
+        <v>309</v>
       </c>
       <c r="H62" t="s">
-        <v>484</v>
+        <v>478</v>
       </c>
     </row>
     <row r="63" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
+        <v>352</v>
+      </c>
+      <c r="B63" t="s">
+        <v>353</v>
+      </c>
+      <c r="C63" t="s">
         <v>354</v>
       </c>
-      <c r="B63" t="s">
+      <c r="D63" t="s">
         <v>355</v>
       </c>
-      <c r="C63" t="s">
+      <c r="E63" t="s">
+        <v>170</v>
+      </c>
+      <c r="F63" t="s">
         <v>356</v>
       </c>
-      <c r="D63" t="s">
+      <c r="G63" t="s">
         <v>357</v>
       </c>
-      <c r="E63" t="s">
-        <v>171</v>
-      </c>
-      <c r="F63" t="s">
+      <c r="H63" t="s">
         <v>358</v>
-      </c>
-      <c r="G63" t="s">
-        <v>359</v>
-      </c>
-      <c r="H63" t="s">
-        <v>360</v>
       </c>
     </row>
     <row r="64" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
+        <v>359</v>
+      </c>
+      <c r="B64" t="s">
+        <v>360</v>
+      </c>
+      <c r="C64" t="s">
         <v>361</v>
       </c>
-      <c r="B64" t="s">
+      <c r="D64" t="s">
         <v>362</v>
       </c>
-      <c r="C64" t="s">
+      <c r="E64" t="s">
+        <v>170</v>
+      </c>
+      <c r="F64" t="s">
         <v>363</v>
       </c>
-      <c r="D64" t="s">
+      <c r="G64" t="s">
         <v>364</v>
       </c>
-      <c r="E64" t="s">
-        <v>171</v>
-      </c>
-      <c r="F64" t="s">
+      <c r="H64" t="s">
         <v>365</v>
-      </c>
-      <c r="G64" t="s">
-        <v>366</v>
-      </c>
-      <c r="H64" t="s">
-        <v>367</v>
       </c>
     </row>
     <row r="65" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
+        <v>366</v>
+      </c>
+      <c r="B65" t="s">
+        <v>367</v>
+      </c>
+      <c r="C65" t="s">
         <v>368</v>
       </c>
-      <c r="B65" t="s">
+      <c r="D65" t="s">
         <v>369</v>
       </c>
-      <c r="C65" t="s">
+      <c r="E65" t="s">
+        <v>170</v>
+      </c>
+      <c r="F65" t="s">
         <v>370</v>
       </c>
-      <c r="D65" t="s">
+      <c r="G65" t="s">
         <v>371</v>
       </c>
-      <c r="E65" t="s">
-        <v>171</v>
-      </c>
-      <c r="F65" t="s">
+      <c r="H65" t="s">
         <v>372</v>
-      </c>
-      <c r="G65" t="s">
-        <v>373</v>
-      </c>
-      <c r="H65" t="s">
-        <v>374</v>
       </c>
     </row>
     <row r="66" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
+        <v>373</v>
+      </c>
+      <c r="B66" t="s">
+        <v>374</v>
+      </c>
+      <c r="C66" t="s">
         <v>375</v>
       </c>
-      <c r="B66" t="s">
+      <c r="D66" t="s">
         <v>376</v>
       </c>
-      <c r="C66" t="s">
+      <c r="E66" t="s">
+        <v>170</v>
+      </c>
+      <c r="F66" t="s">
         <v>377</v>
       </c>
-      <c r="D66" t="s">
+      <c r="G66" t="s">
         <v>378</v>
       </c>
-      <c r="E66" t="s">
-        <v>171</v>
-      </c>
-      <c r="F66" t="s">
-        <v>379</v>
-      </c>
-      <c r="G66" t="s">
-        <v>380</v>
-      </c>
       <c r="H66" t="s">
-        <v>485</v>
+        <v>479</v>
       </c>
     </row>
     <row r="67" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
+        <v>379</v>
+      </c>
+      <c r="B67" t="s">
+        <v>380</v>
+      </c>
+      <c r="C67" t="s">
         <v>381</v>
       </c>
-      <c r="B67" t="s">
+      <c r="D67" t="s">
         <v>382</v>
-      </c>
-      <c r="C67" t="s">
-        <v>383</v>
-      </c>
-      <c r="D67" t="s">
-        <v>384</v>
       </c>
       <c r="E67" t="s">
         <v>82</v>
       </c>
       <c r="F67" t="s">
-        <v>310</v>
+        <v>308</v>
       </c>
       <c r="G67" t="s">
-        <v>311</v>
+        <v>309</v>
       </c>
       <c r="H67" t="s">
-        <v>385</v>
+        <v>383</v>
       </c>
     </row>
     <row r="68" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
+        <v>384</v>
+      </c>
+      <c r="B68" t="s">
+        <v>385</v>
+      </c>
+      <c r="C68" t="s">
         <v>386</v>
       </c>
-      <c r="B68" t="s">
+      <c r="D68" t="s">
         <v>387</v>
-      </c>
-      <c r="C68" t="s">
-        <v>388</v>
-      </c>
-      <c r="D68" t="s">
-        <v>389</v>
       </c>
       <c r="E68" t="s">
         <v>82</v>
       </c>
       <c r="F68" t="s">
+        <v>388</v>
+      </c>
+      <c r="G68" t="s">
+        <v>389</v>
+      </c>
+      <c r="H68" t="s">
         <v>390</v>
-      </c>
-      <c r="G68" t="s">
-        <v>391</v>
-      </c>
-      <c r="H68" t="s">
-        <v>392</v>
       </c>
     </row>
     <row r="69" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
+        <v>391</v>
+      </c>
+      <c r="B69" t="s">
+        <v>392</v>
+      </c>
+      <c r="C69" t="s">
         <v>393</v>
       </c>
-      <c r="B69" t="s">
+      <c r="D69" t="s">
         <v>394</v>
       </c>
-      <c r="C69" t="s">
-        <v>395</v>
-      </c>
-      <c r="D69" t="s">
-        <v>396</v>
-      </c>
       <c r="E69" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="F69" t="s">
-        <v>310</v>
+        <v>308</v>
       </c>
       <c r="G69" t="s">
-        <v>311</v>
+        <v>309</v>
       </c>
       <c r="H69" t="s">
-        <v>486</v>
+        <v>480</v>
       </c>
     </row>
     <row r="70" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
+        <v>395</v>
+      </c>
+      <c r="B70" t="s">
+        <v>396</v>
+      </c>
+      <c r="C70" t="s">
         <v>397</v>
       </c>
-      <c r="B70" t="s">
+      <c r="D70" t="s">
         <v>398</v>
       </c>
-      <c r="C70" t="s">
-        <v>399</v>
-      </c>
-      <c r="D70" t="s">
-        <v>400</v>
-      </c>
       <c r="E70" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="F70" t="s">
-        <v>310</v>
+        <v>308</v>
       </c>
       <c r="G70" t="s">
-        <v>311</v>
+        <v>309</v>
       </c>
       <c r="H70" t="s">
-        <v>487</v>
+        <v>481</v>
       </c>
     </row>
     <row r="71" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
+        <v>399</v>
+      </c>
+      <c r="B71" t="s">
+        <v>495</v>
+      </c>
+      <c r="C71" t="s">
+        <v>400</v>
+      </c>
+      <c r="D71" t="s">
         <v>401</v>
-      </c>
-      <c r="B71" t="s">
-        <v>402</v>
-      </c>
-      <c r="C71" t="s">
-        <v>403</v>
-      </c>
-      <c r="D71" t="s">
-        <v>404</v>
       </c>
       <c r="E71" t="s">
         <v>25</v>
       </c>
       <c r="F71" t="s">
-        <v>405</v>
+        <v>402</v>
       </c>
       <c r="G71" t="s">
         <v>51</v>
       </c>
       <c r="H71" t="s">
-        <v>406</v>
+        <v>403</v>
       </c>
     </row>
     <row r="72" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
+        <v>404</v>
+      </c>
+      <c r="B72" t="s">
+        <v>405</v>
+      </c>
+      <c r="C72" t="s">
+        <v>406</v>
+      </c>
+      <c r="D72" t="s">
         <v>407</v>
-      </c>
-      <c r="B72" t="s">
-        <v>408</v>
-      </c>
-      <c r="C72" t="s">
-        <v>409</v>
-      </c>
-      <c r="D72" t="s">
-        <v>410</v>
       </c>
       <c r="E72" t="s">
         <v>25</v>
@@ -3673,151 +3697,151 @@
         <v>20</v>
       </c>
       <c r="H72" t="s">
-        <v>411</v>
+        <v>408</v>
       </c>
     </row>
     <row r="73" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
-        <v>412</v>
+        <v>409</v>
       </c>
       <c r="B73" t="s">
-        <v>413</v>
+        <v>496</v>
       </c>
       <c r="C73" t="s">
-        <v>414</v>
+        <v>410</v>
       </c>
       <c r="D73" t="s">
-        <v>415</v>
+        <v>411</v>
       </c>
       <c r="E73" t="s">
         <v>25</v>
       </c>
       <c r="F73" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
       <c r="G73" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="H73" t="s">
-        <v>416</v>
+        <v>412</v>
       </c>
     </row>
     <row r="74" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
-        <v>417</v>
+        <v>413</v>
       </c>
       <c r="B74" t="s">
-        <v>418</v>
+        <v>414</v>
       </c>
       <c r="C74" t="s">
-        <v>419</v>
+        <v>415</v>
       </c>
       <c r="D74" t="s">
-        <v>420</v>
+        <v>416</v>
       </c>
       <c r="E74" t="s">
         <v>25</v>
       </c>
       <c r="F74" t="s">
-        <v>421</v>
+        <v>417</v>
       </c>
       <c r="G74" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="H74" t="s">
-        <v>422</v>
+        <v>418</v>
       </c>
     </row>
     <row r="75" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
-        <v>423</v>
+        <v>419</v>
       </c>
       <c r="B75" t="s">
-        <v>424</v>
+        <v>497</v>
       </c>
       <c r="C75" t="s">
-        <v>425</v>
+        <v>420</v>
       </c>
       <c r="D75" t="s">
-        <v>426</v>
+        <v>421</v>
       </c>
       <c r="E75" t="s">
         <v>25</v>
       </c>
       <c r="F75" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="G75" t="s">
         <v>51</v>
       </c>
       <c r="H75" t="s">
-        <v>427</v>
+        <v>422</v>
       </c>
     </row>
     <row r="76" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
-        <v>428</v>
+        <v>423</v>
       </c>
       <c r="B76" t="s">
-        <v>429</v>
+        <v>498</v>
       </c>
       <c r="C76" t="s">
-        <v>430</v>
+        <v>424</v>
       </c>
       <c r="D76" t="s">
-        <v>431</v>
+        <v>425</v>
       </c>
       <c r="E76" t="s">
         <v>25</v>
       </c>
       <c r="F76" t="s">
-        <v>432</v>
+        <v>426</v>
       </c>
       <c r="G76" t="s">
-        <v>311</v>
+        <v>309</v>
       </c>
       <c r="H76" t="s">
-        <v>433</v>
+        <v>427</v>
       </c>
     </row>
     <row r="77" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
-        <v>434</v>
+        <v>428</v>
       </c>
       <c r="B77" t="s">
-        <v>435</v>
+        <v>429</v>
       </c>
       <c r="C77" t="s">
-        <v>436</v>
+        <v>430</v>
       </c>
       <c r="D77" t="s">
-        <v>437</v>
+        <v>431</v>
       </c>
       <c r="E77" t="s">
-        <v>438</v>
+        <v>432</v>
       </c>
       <c r="F77" t="s">
-        <v>439</v>
+        <v>433</v>
       </c>
       <c r="G77" t="s">
         <v>20</v>
       </c>
       <c r="H77" t="s">
-        <v>440</v>
+        <v>434</v>
       </c>
     </row>
     <row r="78" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
-        <v>441</v>
+        <v>435</v>
       </c>
       <c r="B78" t="s">
-        <v>442</v>
+        <v>436</v>
       </c>
       <c r="C78" t="s">
-        <v>443</v>
+        <v>437</v>
       </c>
       <c r="D78" t="s">
-        <v>444</v>
+        <v>438</v>
       </c>
       <c r="E78" t="s">
         <v>43</v>
@@ -3829,85 +3853,111 @@
         <v>31</v>
       </c>
       <c r="H78" t="s">
-        <v>488</v>
+        <v>482</v>
       </c>
     </row>
     <row r="79" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
-        <v>445</v>
+        <v>439</v>
       </c>
       <c r="B79" t="s">
-        <v>446</v>
+        <v>440</v>
       </c>
       <c r="C79" t="s">
-        <v>447</v>
+        <v>441</v>
       </c>
       <c r="D79" t="s">
-        <v>448</v>
+        <v>442</v>
       </c>
       <c r="E79" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="F79" t="s">
-        <v>449</v>
+        <v>443</v>
       </c>
       <c r="G79" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="H79" t="s">
-        <v>450</v>
+        <v>444</v>
       </c>
     </row>
     <row r="80" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
-        <v>451</v>
+        <v>445</v>
       </c>
       <c r="B80" t="s">
-        <v>452</v>
+        <v>446</v>
       </c>
       <c r="C80" t="s">
-        <v>453</v>
+        <v>447</v>
       </c>
       <c r="D80" t="s">
-        <v>454</v>
+        <v>448</v>
       </c>
       <c r="E80" t="s">
         <v>82</v>
       </c>
       <c r="F80" t="s">
-        <v>455</v>
+        <v>449</v>
       </c>
       <c r="G80" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="H80" s="2" t="s">
-        <v>496</v>
+        <v>490</v>
       </c>
     </row>
     <row r="81" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
-        <v>489</v>
+        <v>483</v>
       </c>
       <c r="B81" t="s">
-        <v>490</v>
+        <v>484</v>
       </c>
       <c r="C81" s="2" t="s">
-        <v>491</v>
+        <v>485</v>
       </c>
       <c r="D81" s="2" t="s">
-        <v>493</v>
+        <v>487</v>
       </c>
       <c r="E81" t="s">
         <v>18</v>
       </c>
       <c r="F81" s="2" t="s">
-        <v>494</v>
+        <v>488</v>
       </c>
       <c r="G81" s="2" t="s">
-        <v>495</v>
+        <v>489</v>
       </c>
       <c r="H81" s="2" t="s">
-        <v>497</v>
+        <v>491</v>
+      </c>
+    </row>
+    <row r="82" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A82" t="s">
+        <v>501</v>
+      </c>
+      <c r="B82" t="s">
+        <v>492</v>
+      </c>
+      <c r="C82" s="2" t="s">
+        <v>502</v>
+      </c>
+      <c r="D82" s="2" t="s">
+        <v>503</v>
+      </c>
+      <c r="E82" t="s">
+        <v>146</v>
+      </c>
+      <c r="F82" s="2" t="s">
+        <v>499</v>
+      </c>
+      <c r="G82" s="2" t="s">
+        <v>499</v>
+      </c>
+      <c r="H82" s="2" t="s">
+        <v>500</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update REITs map data for 20260521
</commit_message>
<xml_diff>
--- a/REITs_location_updating.xlsx
+++ b/REITs_location_updating.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\21076\Desktop\公募REITs地图项目\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E3C398FA-7EAF-4E12-AD9A-5AAC70C714F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0C510B4E-6043-410C-94C5-55E5AFC44274}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -579,9 +579,6 @@
     <t>厦门安居集团有限公司</t>
   </si>
   <si>
-    <t>园博公寓,珩琦公寓</t>
-  </si>
-  <si>
     <t>厦门市</t>
   </si>
   <si>
@@ -1426,9 +1423,6 @@
   </si>
   <si>
     <t>{普洛斯北京空港物流园}|{普洛斯增城物流园，普洛斯广州保税物流园，普洛斯江门鹤山物流园}|{普洛斯 (重庆) 城市配送物流中心}|{苏州望亭普洛斯物流园}|{普洛斯淀山湖物流园，普洛斯通州光机电物流园}|{普洛斯顺德物流园}|{普洛斯青岛前湾港国际物流园}</t>
-  </si>
-  <si>
-    <t>{园博公寓，珩琦公寓}</t>
   </si>
   <si>
     <t>{光机电项目，文龙家园项目，朗悦嘉园项目，温泉凯盛家园项目，熙悦尚郡项目，盛悦家园项目}</t>
@@ -1549,6 +1543,14 @@
   </si>
   <si>
     <t>滟澜新宸项目，国瑞熙院项目，未来融尚家园项目</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>园博公寓,珩琦公寓,林边公寓,仁和公寓</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>{园博公寓，珩琦公寓，林边公寓，仁和公寓}</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
@@ -1567,6 +1569,7 @@
       <sz val="11"/>
       <color theme="1"/>
       <name val="宋体"/>
+      <family val="3"/>
       <charset val="134"/>
     </font>
     <font>
@@ -1877,7 +1880,7 @@
         <v>13</v>
       </c>
       <c r="H2" t="s">
-        <v>450</v>
+        <v>449</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
@@ -1903,7 +1906,7 @@
         <v>20</v>
       </c>
       <c r="H3" t="s">
-        <v>451</v>
+        <v>450</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
@@ -1955,7 +1958,7 @@
         <v>31</v>
       </c>
       <c r="H5" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
@@ -2007,7 +2010,7 @@
         <v>45</v>
       </c>
       <c r="H7" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
@@ -2111,7 +2114,7 @@
         <v>57</v>
       </c>
       <c r="H11" t="s">
-        <v>454</v>
+        <v>453</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.25">
@@ -2137,7 +2140,7 @@
         <v>31</v>
       </c>
       <c r="H12" t="s">
-        <v>455</v>
+        <v>454</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
@@ -2163,7 +2166,7 @@
         <v>13</v>
       </c>
       <c r="H13" t="s">
-        <v>456</v>
+        <v>455</v>
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.25">
@@ -2223,7 +2226,7 @@
         <v>91</v>
       </c>
       <c r="B16" t="s">
-        <v>493</v>
+        <v>491</v>
       </c>
       <c r="C16" t="s">
         <v>92</v>
@@ -2293,7 +2296,7 @@
         <v>102</v>
       </c>
       <c r="H18" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.25">
@@ -2319,7 +2322,7 @@
         <v>13</v>
       </c>
       <c r="H19" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.25">
@@ -2345,7 +2348,7 @@
         <v>117</v>
       </c>
       <c r="H20" t="s">
-        <v>459</v>
+        <v>458</v>
       </c>
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.25">
@@ -2397,7 +2400,7 @@
         <v>130</v>
       </c>
       <c r="H22" t="s">
-        <v>460</v>
+        <v>459</v>
       </c>
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.25">
@@ -2423,7 +2426,7 @@
         <v>130</v>
       </c>
       <c r="H23" t="s">
-        <v>461</v>
+        <v>460</v>
       </c>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.25">
@@ -2449,7 +2452,7 @@
         <v>141</v>
       </c>
       <c r="H24" t="s">
-        <v>462</v>
+        <v>461</v>
       </c>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.25">
@@ -2475,7 +2478,7 @@
         <v>13</v>
       </c>
       <c r="H25" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.25">
@@ -2579,7 +2582,7 @@
         <v>13</v>
       </c>
       <c r="H29" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
     </row>
     <row r="30" spans="1:8" x14ac:dyDescent="0.25">
@@ -2605,7 +2608,7 @@
         <v>13</v>
       </c>
       <c r="H30" t="s">
-        <v>465</v>
+        <v>464</v>
       </c>
     </row>
     <row r="31" spans="1:8" x14ac:dyDescent="0.25">
@@ -2631,7 +2634,7 @@
         <v>180</v>
       </c>
       <c r="H31" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
     </row>
     <row r="32" spans="1:8" x14ac:dyDescent="0.25">
@@ -2644,37 +2647,37 @@
       <c r="C32" t="s">
         <v>183</v>
       </c>
-      <c r="D32" t="s">
-        <v>184</v>
+      <c r="D32" s="2" t="s">
+        <v>502</v>
       </c>
       <c r="E32" t="s">
         <v>146</v>
       </c>
       <c r="F32" t="s">
+        <v>184</v>
+      </c>
+      <c r="G32" t="s">
         <v>185</v>
       </c>
-      <c r="G32" t="s">
-        <v>186</v>
-      </c>
-      <c r="H32" t="s">
-        <v>467</v>
+      <c r="H32" s="2" t="s">
+        <v>503</v>
       </c>
     </row>
     <row r="33" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
+        <v>186</v>
+      </c>
+      <c r="B33" t="s">
         <v>187</v>
       </c>
-      <c r="B33" t="s">
+      <c r="C33" t="s">
         <v>188</v>
       </c>
-      <c r="C33" t="s">
+      <c r="D33" t="s">
         <v>189</v>
       </c>
-      <c r="D33" t="s">
+      <c r="E33" t="s">
         <v>190</v>
-      </c>
-      <c r="E33" t="s">
-        <v>191</v>
       </c>
       <c r="F33" t="s">
         <v>129</v>
@@ -2683,21 +2686,21 @@
         <v>130</v>
       </c>
       <c r="H33" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
     </row>
     <row r="34" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
+        <v>192</v>
+      </c>
+      <c r="B34" t="s">
         <v>193</v>
       </c>
-      <c r="B34" t="s">
+      <c r="C34" t="s">
         <v>194</v>
       </c>
-      <c r="C34" t="s">
+      <c r="D34" t="s">
         <v>195</v>
-      </c>
-      <c r="D34" t="s">
-        <v>196</v>
       </c>
       <c r="E34" t="s">
         <v>18</v>
@@ -2709,21 +2712,21 @@
         <v>130</v>
       </c>
       <c r="H34" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
     </row>
     <row r="35" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
+        <v>197</v>
+      </c>
+      <c r="B35" t="s">
         <v>198</v>
       </c>
-      <c r="B35" t="s">
+      <c r="C35" t="s">
         <v>199</v>
       </c>
-      <c r="C35" t="s">
+      <c r="D35" t="s">
         <v>200</v>
-      </c>
-      <c r="D35" t="s">
-        <v>201</v>
       </c>
       <c r="E35" t="s">
         <v>146</v>
@@ -2735,47 +2738,47 @@
         <v>31</v>
       </c>
       <c r="H35" t="s">
-        <v>468</v>
+        <v>466</v>
       </c>
     </row>
     <row r="36" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
+        <v>201</v>
+      </c>
+      <c r="B36" t="s">
         <v>202</v>
       </c>
-      <c r="B36" t="s">
+      <c r="C36" t="s">
         <v>203</v>
       </c>
-      <c r="C36" t="s">
+      <c r="D36" t="s">
         <v>204</v>
-      </c>
-      <c r="D36" t="s">
-        <v>205</v>
       </c>
       <c r="E36" t="s">
         <v>18</v>
       </c>
       <c r="F36" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="G36" t="s">
         <v>130</v>
       </c>
       <c r="H36" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
     </row>
     <row r="37" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
+        <v>207</v>
+      </c>
+      <c r="B37" t="s">
         <v>208</v>
       </c>
-      <c r="B37" t="s">
+      <c r="C37" t="s">
         <v>209</v>
       </c>
-      <c r="C37" t="s">
+      <c r="D37" t="s">
         <v>210</v>
-      </c>
-      <c r="D37" t="s">
-        <v>211</v>
       </c>
       <c r="E37" t="s">
         <v>146</v>
@@ -2787,21 +2790,21 @@
         <v>13</v>
       </c>
       <c r="H37" t="s">
-        <v>469</v>
+        <v>467</v>
       </c>
     </row>
     <row r="38" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
+        <v>211</v>
+      </c>
+      <c r="B38" t="s">
         <v>212</v>
       </c>
-      <c r="B38" t="s">
+      <c r="C38" t="s">
         <v>213</v>
       </c>
-      <c r="C38" t="s">
+      <c r="D38" t="s">
         <v>214</v>
-      </c>
-      <c r="D38" t="s">
-        <v>215</v>
       </c>
       <c r="E38" t="s">
         <v>170</v>
@@ -2813,21 +2816,21 @@
         <v>130</v>
       </c>
       <c r="H38" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
     </row>
     <row r="39" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
+        <v>216</v>
+      </c>
+      <c r="B39" t="s">
         <v>217</v>
       </c>
-      <c r="B39" t="s">
+      <c r="C39" t="s">
         <v>218</v>
       </c>
-      <c r="C39" t="s">
+      <c r="D39" t="s">
         <v>219</v>
-      </c>
-      <c r="D39" t="s">
-        <v>220</v>
       </c>
       <c r="E39" t="s">
         <v>12</v>
@@ -2839,47 +2842,47 @@
         <v>31</v>
       </c>
       <c r="H39" t="s">
-        <v>470</v>
+        <v>468</v>
       </c>
     </row>
     <row r="40" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
+        <v>220</v>
+      </c>
+      <c r="B40" t="s">
         <v>221</v>
       </c>
-      <c r="B40" t="s">
+      <c r="C40" t="s">
         <v>222</v>
       </c>
-      <c r="C40" t="s">
+      <c r="D40" t="s">
         <v>223</v>
-      </c>
-      <c r="D40" t="s">
-        <v>224</v>
       </c>
       <c r="E40" t="s">
         <v>25</v>
       </c>
       <c r="F40" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="G40" t="s">
         <v>20</v>
       </c>
       <c r="H40" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
     </row>
     <row r="41" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
+        <v>226</v>
+      </c>
+      <c r="B41" t="s">
         <v>227</v>
       </c>
-      <c r="B41" t="s">
+      <c r="C41" t="s">
         <v>228</v>
       </c>
-      <c r="C41" t="s">
+      <c r="D41" t="s">
         <v>229</v>
-      </c>
-      <c r="D41" t="s">
-        <v>230</v>
       </c>
       <c r="E41" t="s">
         <v>170</v>
@@ -2891,21 +2894,21 @@
         <v>102</v>
       </c>
       <c r="H41" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
     </row>
     <row r="42" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
+        <v>231</v>
+      </c>
+      <c r="B42" t="s">
         <v>232</v>
       </c>
-      <c r="B42" t="s">
+      <c r="C42" t="s">
         <v>233</v>
       </c>
-      <c r="C42" t="s">
+      <c r="D42" t="s">
         <v>234</v>
-      </c>
-      <c r="D42" t="s">
-        <v>235</v>
       </c>
       <c r="E42" t="s">
         <v>146</v>
@@ -2917,177 +2920,177 @@
         <v>130</v>
       </c>
       <c r="H42" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
     </row>
     <row r="43" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
+        <v>236</v>
+      </c>
+      <c r="B43" t="s">
         <v>237</v>
       </c>
-      <c r="B43" t="s">
+      <c r="C43" t="s">
         <v>238</v>
       </c>
-      <c r="C43" t="s">
+      <c r="D43" t="s">
         <v>239</v>
-      </c>
-      <c r="D43" t="s">
-        <v>240</v>
       </c>
       <c r="E43" t="s">
         <v>18</v>
       </c>
       <c r="F43" t="s">
+        <v>240</v>
+      </c>
+      <c r="G43" t="s">
         <v>241</v>
       </c>
-      <c r="G43" t="s">
+      <c r="H43" t="s">
         <v>242</v>
-      </c>
-      <c r="H43" t="s">
-        <v>243</v>
       </c>
     </row>
     <row r="44" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
+        <v>243</v>
+      </c>
+      <c r="B44" t="s">
         <v>244</v>
       </c>
-      <c r="B44" t="s">
+      <c r="C44" t="s">
         <v>245</v>
       </c>
-      <c r="C44" t="s">
+      <c r="D44" t="s">
         <v>246</v>
       </c>
-      <c r="D44" t="s">
+      <c r="E44" t="s">
         <v>247</v>
       </c>
-      <c r="E44" t="s">
+      <c r="F44" t="s">
         <v>248</v>
-      </c>
-      <c r="F44" t="s">
-        <v>249</v>
       </c>
       <c r="G44" t="s">
         <v>51</v>
       </c>
       <c r="H44" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
     </row>
     <row r="45" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
+        <v>250</v>
+      </c>
+      <c r="B45" t="s">
         <v>251</v>
       </c>
-      <c r="B45" t="s">
+      <c r="C45" t="s">
         <v>252</v>
       </c>
-      <c r="C45" t="s">
+      <c r="D45" t="s">
         <v>253</v>
-      </c>
-      <c r="D45" t="s">
-        <v>254</v>
       </c>
       <c r="E45" t="s">
         <v>12</v>
       </c>
       <c r="F45" t="s">
+        <v>254</v>
+      </c>
+      <c r="G45" t="s">
         <v>255</v>
       </c>
-      <c r="G45" t="s">
+      <c r="H45" t="s">
         <v>256</v>
-      </c>
-      <c r="H45" t="s">
-        <v>257</v>
       </c>
     </row>
     <row r="46" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
+        <v>257</v>
+      </c>
+      <c r="B46" t="s">
         <v>258</v>
       </c>
-      <c r="B46" t="s">
+      <c r="C46" t="s">
         <v>259</v>
       </c>
-      <c r="C46" t="s">
+      <c r="D46" t="s">
         <v>260</v>
-      </c>
-      <c r="D46" t="s">
-        <v>261</v>
       </c>
       <c r="E46" t="s">
         <v>82</v>
       </c>
       <c r="F46" t="s">
+        <v>261</v>
+      </c>
+      <c r="G46" t="s">
         <v>262</v>
       </c>
-      <c r="G46" t="s">
+      <c r="H46" t="s">
         <v>263</v>
-      </c>
-      <c r="H46" t="s">
-        <v>264</v>
       </c>
     </row>
     <row r="47" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
+        <v>264</v>
+      </c>
+      <c r="B47" t="s">
         <v>265</v>
       </c>
-      <c r="B47" t="s">
+      <c r="C47" t="s">
         <v>266</v>
       </c>
-      <c r="C47" t="s">
+      <c r="D47" t="s">
         <v>267</v>
-      </c>
-      <c r="D47" t="s">
-        <v>268</v>
       </c>
       <c r="E47" t="s">
         <v>170</v>
       </c>
       <c r="F47" t="s">
+        <v>268</v>
+      </c>
+      <c r="G47" t="s">
         <v>269</v>
       </c>
-      <c r="G47" t="s">
-        <v>270</v>
-      </c>
       <c r="H47" t="s">
-        <v>471</v>
+        <v>469</v>
       </c>
     </row>
     <row r="48" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
+        <v>270</v>
+      </c>
+      <c r="B48" t="s">
+        <v>492</v>
+      </c>
+      <c r="C48" t="s">
         <v>271</v>
       </c>
-      <c r="B48" t="s">
-        <v>494</v>
-      </c>
-      <c r="C48" t="s">
+      <c r="D48" t="s">
         <v>272</v>
-      </c>
-      <c r="D48" t="s">
-        <v>273</v>
       </c>
       <c r="E48" t="s">
         <v>25</v>
       </c>
       <c r="F48" t="s">
+        <v>273</v>
+      </c>
+      <c r="G48" t="s">
         <v>274</v>
       </c>
-      <c r="G48" t="s">
+      <c r="H48" t="s">
         <v>275</v>
-      </c>
-      <c r="H48" t="s">
-        <v>276</v>
       </c>
     </row>
     <row r="49" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
+        <v>276</v>
+      </c>
+      <c r="B49" t="s">
         <v>277</v>
       </c>
-      <c r="B49" t="s">
+      <c r="C49" t="s">
         <v>278</v>
       </c>
-      <c r="C49" t="s">
+      <c r="D49" t="s">
         <v>279</v>
-      </c>
-      <c r="D49" t="s">
-        <v>280</v>
       </c>
       <c r="E49" t="s">
         <v>12</v>
@@ -3099,99 +3102,99 @@
         <v>31</v>
       </c>
       <c r="H49" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
     </row>
     <row r="50" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
+        <v>281</v>
+      </c>
+      <c r="B50" t="s">
         <v>282</v>
       </c>
-      <c r="B50" t="s">
+      <c r="C50" t="s">
         <v>283</v>
       </c>
-      <c r="C50" t="s">
+      <c r="D50" t="s">
         <v>284</v>
-      </c>
-      <c r="D50" t="s">
-        <v>285</v>
       </c>
       <c r="E50" t="s">
         <v>82</v>
       </c>
       <c r="F50" t="s">
+        <v>285</v>
+      </c>
+      <c r="G50" t="s">
         <v>286</v>
       </c>
-      <c r="G50" t="s">
-        <v>287</v>
-      </c>
       <c r="H50" t="s">
-        <v>472</v>
+        <v>470</v>
       </c>
     </row>
     <row r="51" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
+        <v>287</v>
+      </c>
+      <c r="B51" t="s">
         <v>288</v>
       </c>
-      <c r="B51" t="s">
+      <c r="C51" t="s">
         <v>289</v>
       </c>
-      <c r="C51" t="s">
+      <c r="D51" t="s">
         <v>290</v>
-      </c>
-      <c r="D51" t="s">
-        <v>291</v>
       </c>
       <c r="E51" t="s">
         <v>12</v>
       </c>
       <c r="F51" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="G51" t="s">
         <v>130</v>
       </c>
       <c r="H51" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
     </row>
     <row r="52" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
+        <v>292</v>
+      </c>
+      <c r="B52" t="s">
         <v>293</v>
       </c>
-      <c r="B52" t="s">
+      <c r="C52" t="s">
         <v>294</v>
       </c>
-      <c r="C52" t="s">
+      <c r="D52" t="s">
         <v>295</v>
-      </c>
-      <c r="D52" t="s">
-        <v>296</v>
       </c>
       <c r="E52" t="s">
         <v>170</v>
       </c>
       <c r="F52" t="s">
+        <v>296</v>
+      </c>
+      <c r="G52" t="s">
         <v>297</v>
       </c>
-      <c r="G52" t="s">
+      <c r="H52" t="s">
         <v>298</v>
-      </c>
-      <c r="H52" t="s">
-        <v>299</v>
       </c>
     </row>
     <row r="53" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
+        <v>299</v>
+      </c>
+      <c r="B53" t="s">
         <v>300</v>
       </c>
-      <c r="B53" t="s">
+      <c r="C53" t="s">
         <v>301</v>
       </c>
-      <c r="C53" t="s">
+      <c r="D53" t="s">
         <v>302</v>
-      </c>
-      <c r="D53" t="s">
-        <v>303</v>
       </c>
       <c r="E53" t="s">
         <v>12</v>
@@ -3203,73 +3206,73 @@
         <v>31</v>
       </c>
       <c r="H53" t="s">
-        <v>473</v>
+        <v>471</v>
       </c>
     </row>
     <row r="54" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
+        <v>303</v>
+      </c>
+      <c r="B54" t="s">
         <v>304</v>
       </c>
-      <c r="B54" t="s">
+      <c r="C54" t="s">
         <v>305</v>
       </c>
-      <c r="C54" t="s">
+      <c r="D54" t="s">
         <v>306</v>
-      </c>
-      <c r="D54" t="s">
-        <v>307</v>
       </c>
       <c r="E54" t="s">
         <v>12</v>
       </c>
       <c r="F54" t="s">
+        <v>307</v>
+      </c>
+      <c r="G54" t="s">
         <v>308</v>
       </c>
-      <c r="G54" t="s">
-        <v>309</v>
-      </c>
       <c r="H54" t="s">
-        <v>474</v>
+        <v>472</v>
       </c>
     </row>
     <row r="55" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
+        <v>309</v>
+      </c>
+      <c r="B55" t="s">
         <v>310</v>
       </c>
-      <c r="B55" t="s">
+      <c r="C55" t="s">
         <v>311</v>
       </c>
-      <c r="C55" t="s">
+      <c r="D55" t="s">
         <v>312</v>
-      </c>
-      <c r="D55" t="s">
-        <v>313</v>
       </c>
       <c r="E55" t="s">
         <v>12</v>
       </c>
       <c r="F55" t="s">
+        <v>313</v>
+      </c>
+      <c r="G55" t="s">
         <v>314</v>
       </c>
-      <c r="G55" t="s">
+      <c r="H55" t="s">
         <v>315</v>
-      </c>
-      <c r="H55" t="s">
-        <v>316</v>
       </c>
     </row>
     <row r="56" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
+        <v>316</v>
+      </c>
+      <c r="B56" t="s">
         <v>317</v>
       </c>
-      <c r="B56" t="s">
+      <c r="C56" t="s">
         <v>318</v>
       </c>
-      <c r="C56" t="s">
-        <v>319</v>
-      </c>
       <c r="D56" s="2" t="s">
-        <v>486</v>
+        <v>484</v>
       </c>
       <c r="E56" t="s">
         <v>12</v>
@@ -3281,411 +3284,411 @@
         <v>20</v>
       </c>
       <c r="H56" t="s">
-        <v>475</v>
+        <v>473</v>
       </c>
     </row>
     <row r="57" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
+        <v>319</v>
+      </c>
+      <c r="B57" t="s">
         <v>320</v>
       </c>
-      <c r="B57" t="s">
+      <c r="C57" t="s">
         <v>321</v>
       </c>
-      <c r="C57" t="s">
+      <c r="D57" t="s">
         <v>322</v>
-      </c>
-      <c r="D57" t="s">
-        <v>323</v>
       </c>
       <c r="E57" t="s">
         <v>12</v>
       </c>
       <c r="F57" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="G57" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="H57" t="s">
-        <v>476</v>
+        <v>474</v>
       </c>
     </row>
     <row r="58" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
+        <v>324</v>
+      </c>
+      <c r="B58" t="s">
         <v>325</v>
       </c>
-      <c r="B58" t="s">
+      <c r="C58" t="s">
         <v>326</v>
       </c>
-      <c r="C58" t="s">
+      <c r="D58" t="s">
         <v>327</v>
-      </c>
-      <c r="D58" t="s">
-        <v>328</v>
       </c>
       <c r="E58" t="s">
         <v>12</v>
       </c>
       <c r="F58" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="G58" t="s">
         <v>123</v>
       </c>
       <c r="H58" t="s">
-        <v>477</v>
+        <v>475</v>
       </c>
     </row>
     <row r="59" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
+        <v>329</v>
+      </c>
+      <c r="B59" t="s">
         <v>330</v>
       </c>
-      <c r="B59" t="s">
+      <c r="C59" t="s">
         <v>331</v>
       </c>
-      <c r="C59" t="s">
+      <c r="D59" t="s">
         <v>332</v>
-      </c>
-      <c r="D59" t="s">
-        <v>333</v>
       </c>
       <c r="E59" t="s">
         <v>18</v>
       </c>
       <c r="F59" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="G59" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="H59" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
     </row>
     <row r="60" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
+        <v>334</v>
+      </c>
+      <c r="B60" t="s">
         <v>335</v>
       </c>
-      <c r="B60" t="s">
+      <c r="C60" t="s">
         <v>336</v>
       </c>
-      <c r="C60" t="s">
+      <c r="D60" t="s">
         <v>337</v>
-      </c>
-      <c r="D60" t="s">
-        <v>338</v>
       </c>
       <c r="E60" t="s">
         <v>18</v>
       </c>
       <c r="F60" t="s">
+        <v>338</v>
+      </c>
+      <c r="G60" t="s">
         <v>339</v>
       </c>
-      <c r="G60" t="s">
+      <c r="H60" t="s">
         <v>340</v>
-      </c>
-      <c r="H60" t="s">
-        <v>341</v>
       </c>
     </row>
     <row r="61" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
+        <v>341</v>
+      </c>
+      <c r="B61" t="s">
         <v>342</v>
       </c>
-      <c r="B61" t="s">
+      <c r="C61" t="s">
         <v>343</v>
       </c>
-      <c r="C61" t="s">
+      <c r="D61" t="s">
         <v>344</v>
-      </c>
-      <c r="D61" t="s">
-        <v>345</v>
       </c>
       <c r="E61" t="s">
         <v>18</v>
       </c>
       <c r="F61" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="G61" t="s">
         <v>64</v>
       </c>
       <c r="H61" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
     </row>
     <row r="62" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
+        <v>347</v>
+      </c>
+      <c r="B62" t="s">
         <v>348</v>
       </c>
-      <c r="B62" t="s">
+      <c r="C62" t="s">
         <v>349</v>
       </c>
-      <c r="C62" t="s">
+      <c r="D62" t="s">
         <v>350</v>
-      </c>
-      <c r="D62" t="s">
-        <v>351</v>
       </c>
       <c r="E62" t="s">
         <v>170</v>
       </c>
       <c r="F62" t="s">
+        <v>307</v>
+      </c>
+      <c r="G62" t="s">
         <v>308</v>
       </c>
-      <c r="G62" t="s">
-        <v>309</v>
-      </c>
       <c r="H62" t="s">
-        <v>478</v>
+        <v>476</v>
       </c>
     </row>
     <row r="63" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
+        <v>351</v>
+      </c>
+      <c r="B63" t="s">
         <v>352</v>
       </c>
-      <c r="B63" t="s">
+      <c r="C63" t="s">
         <v>353</v>
       </c>
-      <c r="C63" t="s">
+      <c r="D63" t="s">
         <v>354</v>
-      </c>
-      <c r="D63" t="s">
-        <v>355</v>
       </c>
       <c r="E63" t="s">
         <v>170</v>
       </c>
       <c r="F63" t="s">
+        <v>355</v>
+      </c>
+      <c r="G63" t="s">
         <v>356</v>
       </c>
-      <c r="G63" t="s">
+      <c r="H63" t="s">
         <v>357</v>
-      </c>
-      <c r="H63" t="s">
-        <v>358</v>
       </c>
     </row>
     <row r="64" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
+        <v>358</v>
+      </c>
+      <c r="B64" t="s">
         <v>359</v>
       </c>
-      <c r="B64" t="s">
+      <c r="C64" t="s">
         <v>360</v>
       </c>
-      <c r="C64" t="s">
+      <c r="D64" t="s">
         <v>361</v>
-      </c>
-      <c r="D64" t="s">
-        <v>362</v>
       </c>
       <c r="E64" t="s">
         <v>170</v>
       </c>
       <c r="F64" t="s">
+        <v>362</v>
+      </c>
+      <c r="G64" t="s">
         <v>363</v>
       </c>
-      <c r="G64" t="s">
+      <c r="H64" t="s">
         <v>364</v>
-      </c>
-      <c r="H64" t="s">
-        <v>365</v>
       </c>
     </row>
     <row r="65" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
+        <v>365</v>
+      </c>
+      <c r="B65" t="s">
         <v>366</v>
       </c>
-      <c r="B65" t="s">
+      <c r="C65" t="s">
         <v>367</v>
       </c>
-      <c r="C65" t="s">
+      <c r="D65" t="s">
         <v>368</v>
-      </c>
-      <c r="D65" t="s">
-        <v>369</v>
       </c>
       <c r="E65" t="s">
         <v>170</v>
       </c>
       <c r="F65" t="s">
+        <v>369</v>
+      </c>
+      <c r="G65" t="s">
         <v>370</v>
       </c>
-      <c r="G65" t="s">
+      <c r="H65" t="s">
         <v>371</v>
-      </c>
-      <c r="H65" t="s">
-        <v>372</v>
       </c>
     </row>
     <row r="66" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
+        <v>372</v>
+      </c>
+      <c r="B66" t="s">
         <v>373</v>
       </c>
-      <c r="B66" t="s">
+      <c r="C66" t="s">
         <v>374</v>
       </c>
-      <c r="C66" t="s">
+      <c r="D66" t="s">
         <v>375</v>
-      </c>
-      <c r="D66" t="s">
-        <v>376</v>
       </c>
       <c r="E66" t="s">
         <v>170</v>
       </c>
       <c r="F66" t="s">
+        <v>376</v>
+      </c>
+      <c r="G66" t="s">
         <v>377</v>
       </c>
-      <c r="G66" t="s">
-        <v>378</v>
-      </c>
       <c r="H66" t="s">
-        <v>479</v>
+        <v>477</v>
       </c>
     </row>
     <row r="67" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
+        <v>378</v>
+      </c>
+      <c r="B67" t="s">
         <v>379</v>
       </c>
-      <c r="B67" t="s">
+      <c r="C67" t="s">
         <v>380</v>
       </c>
-      <c r="C67" t="s">
+      <c r="D67" t="s">
         <v>381</v>
-      </c>
-      <c r="D67" t="s">
-        <v>382</v>
       </c>
       <c r="E67" t="s">
         <v>82</v>
       </c>
       <c r="F67" t="s">
+        <v>307</v>
+      </c>
+      <c r="G67" t="s">
         <v>308</v>
       </c>
-      <c r="G67" t="s">
-        <v>309</v>
-      </c>
       <c r="H67" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
     </row>
     <row r="68" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
+        <v>383</v>
+      </c>
+      <c r="B68" t="s">
         <v>384</v>
       </c>
-      <c r="B68" t="s">
+      <c r="C68" t="s">
         <v>385</v>
       </c>
-      <c r="C68" t="s">
+      <c r="D68" t="s">
         <v>386</v>
-      </c>
-      <c r="D68" t="s">
-        <v>387</v>
       </c>
       <c r="E68" t="s">
         <v>82</v>
       </c>
       <c r="F68" t="s">
+        <v>387</v>
+      </c>
+      <c r="G68" t="s">
         <v>388</v>
       </c>
-      <c r="G68" t="s">
+      <c r="H68" t="s">
         <v>389</v>
-      </c>
-      <c r="H68" t="s">
-        <v>390</v>
       </c>
     </row>
     <row r="69" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
+        <v>390</v>
+      </c>
+      <c r="B69" t="s">
         <v>391</v>
       </c>
-      <c r="B69" t="s">
+      <c r="C69" t="s">
         <v>392</v>
       </c>
-      <c r="C69" t="s">
+      <c r="D69" t="s">
         <v>393</v>
-      </c>
-      <c r="D69" t="s">
-        <v>394</v>
       </c>
       <c r="E69" t="s">
         <v>146</v>
       </c>
       <c r="F69" t="s">
+        <v>307</v>
+      </c>
+      <c r="G69" t="s">
         <v>308</v>
       </c>
-      <c r="G69" t="s">
-        <v>309</v>
-      </c>
       <c r="H69" t="s">
-        <v>480</v>
+        <v>478</v>
       </c>
     </row>
     <row r="70" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
+        <v>394</v>
+      </c>
+      <c r="B70" t="s">
         <v>395</v>
       </c>
-      <c r="B70" t="s">
+      <c r="C70" t="s">
         <v>396</v>
       </c>
-      <c r="C70" t="s">
+      <c r="D70" t="s">
         <v>397</v>
-      </c>
-      <c r="D70" t="s">
-        <v>398</v>
       </c>
       <c r="E70" t="s">
         <v>146</v>
       </c>
       <c r="F70" t="s">
+        <v>307</v>
+      </c>
+      <c r="G70" t="s">
         <v>308</v>
       </c>
-      <c r="G70" t="s">
-        <v>309</v>
-      </c>
       <c r="H70" t="s">
-        <v>481</v>
+        <v>479</v>
       </c>
     </row>
     <row r="71" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
+        <v>398</v>
+      </c>
+      <c r="B71" t="s">
+        <v>493</v>
+      </c>
+      <c r="C71" t="s">
         <v>399</v>
       </c>
-      <c r="B71" t="s">
-        <v>495</v>
-      </c>
-      <c r="C71" t="s">
+      <c r="D71" t="s">
         <v>400</v>
-      </c>
-      <c r="D71" t="s">
-        <v>401</v>
       </c>
       <c r="E71" t="s">
         <v>25</v>
       </c>
       <c r="F71" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="G71" t="s">
         <v>51</v>
       </c>
       <c r="H71" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
     </row>
     <row r="72" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
+        <v>403</v>
+      </c>
+      <c r="B72" t="s">
         <v>404</v>
       </c>
-      <c r="B72" t="s">
+      <c r="C72" t="s">
         <v>405</v>
       </c>
-      <c r="C72" t="s">
+      <c r="D72" t="s">
         <v>406</v>
-      </c>
-      <c r="D72" t="s">
-        <v>407</v>
       </c>
       <c r="E72" t="s">
         <v>25</v>
@@ -3697,151 +3700,151 @@
         <v>20</v>
       </c>
       <c r="H72" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
     </row>
     <row r="73" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
+        <v>408</v>
+      </c>
+      <c r="B73" t="s">
+        <v>494</v>
+      </c>
+      <c r="C73" t="s">
         <v>409</v>
       </c>
-      <c r="B73" t="s">
-        <v>496</v>
-      </c>
-      <c r="C73" t="s">
+      <c r="D73" t="s">
         <v>410</v>
-      </c>
-      <c r="D73" t="s">
-        <v>411</v>
       </c>
       <c r="E73" t="s">
         <v>25</v>
       </c>
       <c r="F73" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="G73" t="s">
         <v>123</v>
       </c>
       <c r="H73" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
     </row>
     <row r="74" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
+        <v>412</v>
+      </c>
+      <c r="B74" t="s">
         <v>413</v>
       </c>
-      <c r="B74" t="s">
+      <c r="C74" t="s">
         <v>414</v>
       </c>
-      <c r="C74" t="s">
+      <c r="D74" t="s">
         <v>415</v>
-      </c>
-      <c r="D74" t="s">
-        <v>416</v>
       </c>
       <c r="E74" t="s">
         <v>25</v>
       </c>
       <c r="F74" t="s">
+        <v>416</v>
+      </c>
+      <c r="G74" t="s">
+        <v>185</v>
+      </c>
+      <c r="H74" t="s">
         <v>417</v>
-      </c>
-      <c r="G74" t="s">
-        <v>186</v>
-      </c>
-      <c r="H74" t="s">
-        <v>418</v>
       </c>
     </row>
     <row r="75" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
+        <v>418</v>
+      </c>
+      <c r="B75" t="s">
+        <v>495</v>
+      </c>
+      <c r="C75" t="s">
         <v>419</v>
       </c>
-      <c r="B75" t="s">
-        <v>497</v>
-      </c>
-      <c r="C75" t="s">
+      <c r="D75" t="s">
         <v>420</v>
-      </c>
-      <c r="D75" t="s">
-        <v>421</v>
       </c>
       <c r="E75" t="s">
         <v>25</v>
       </c>
       <c r="F75" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="G75" t="s">
         <v>51</v>
       </c>
       <c r="H75" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
     </row>
     <row r="76" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
+        <v>422</v>
+      </c>
+      <c r="B76" t="s">
+        <v>496</v>
+      </c>
+      <c r="C76" t="s">
         <v>423</v>
       </c>
-      <c r="B76" t="s">
-        <v>498</v>
-      </c>
-      <c r="C76" t="s">
+      <c r="D76" t="s">
         <v>424</v>
-      </c>
-      <c r="D76" t="s">
-        <v>425</v>
       </c>
       <c r="E76" t="s">
         <v>25</v>
       </c>
       <c r="F76" t="s">
+        <v>425</v>
+      </c>
+      <c r="G76" t="s">
+        <v>308</v>
+      </c>
+      <c r="H76" t="s">
         <v>426</v>
-      </c>
-      <c r="G76" t="s">
-        <v>309</v>
-      </c>
-      <c r="H76" t="s">
-        <v>427</v>
       </c>
     </row>
     <row r="77" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
+        <v>427</v>
+      </c>
+      <c r="B77" t="s">
         <v>428</v>
       </c>
-      <c r="B77" t="s">
+      <c r="C77" t="s">
         <v>429</v>
       </c>
-      <c r="C77" t="s">
+      <c r="D77" t="s">
         <v>430</v>
       </c>
-      <c r="D77" t="s">
+      <c r="E77" t="s">
         <v>431</v>
       </c>
-      <c r="E77" t="s">
+      <c r="F77" t="s">
         <v>432</v>
-      </c>
-      <c r="F77" t="s">
-        <v>433</v>
       </c>
       <c r="G77" t="s">
         <v>20</v>
       </c>
       <c r="H77" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
     </row>
     <row r="78" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
+        <v>434</v>
+      </c>
+      <c r="B78" t="s">
         <v>435</v>
       </c>
-      <c r="B78" t="s">
+      <c r="C78" t="s">
         <v>436</v>
       </c>
-      <c r="C78" t="s">
+      <c r="D78" t="s">
         <v>437</v>
-      </c>
-      <c r="D78" t="s">
-        <v>438</v>
       </c>
       <c r="E78" t="s">
         <v>43</v>
@@ -3853,111 +3856,111 @@
         <v>31</v>
       </c>
       <c r="H78" t="s">
-        <v>482</v>
+        <v>480</v>
       </c>
     </row>
     <row r="79" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
+        <v>438</v>
+      </c>
+      <c r="B79" t="s">
         <v>439</v>
       </c>
-      <c r="B79" t="s">
+      <c r="C79" t="s">
         <v>440</v>
       </c>
-      <c r="C79" t="s">
+      <c r="D79" t="s">
         <v>441</v>
       </c>
-      <c r="D79" t="s">
+      <c r="E79" t="s">
+        <v>190</v>
+      </c>
+      <c r="F79" t="s">
         <v>442</v>
       </c>
-      <c r="E79" t="s">
-        <v>191</v>
-      </c>
-      <c r="F79" t="s">
+      <c r="G79" t="s">
+        <v>241</v>
+      </c>
+      <c r="H79" t="s">
         <v>443</v>
-      </c>
-      <c r="G79" t="s">
-        <v>242</v>
-      </c>
-      <c r="H79" t="s">
-        <v>444</v>
       </c>
     </row>
     <row r="80" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
+        <v>444</v>
+      </c>
+      <c r="B80" t="s">
         <v>445</v>
       </c>
-      <c r="B80" t="s">
+      <c r="C80" t="s">
         <v>446</v>
       </c>
-      <c r="C80" t="s">
+      <c r="D80" t="s">
         <v>447</v>
-      </c>
-      <c r="D80" t="s">
-        <v>448</v>
       </c>
       <c r="E80" t="s">
         <v>82</v>
       </c>
       <c r="F80" t="s">
-        <v>449</v>
+        <v>448</v>
       </c>
       <c r="G80" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="H80" s="2" t="s">
-        <v>490</v>
+        <v>488</v>
       </c>
     </row>
     <row r="81" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
+        <v>481</v>
+      </c>
+      <c r="B81" t="s">
+        <v>482</v>
+      </c>
+      <c r="C81" s="2" t="s">
         <v>483</v>
       </c>
-      <c r="B81" t="s">
-        <v>484</v>
-      </c>
-      <c r="C81" s="2" t="s">
+      <c r="D81" s="2" t="s">
         <v>485</v>
-      </c>
-      <c r="D81" s="2" t="s">
-        <v>487</v>
       </c>
       <c r="E81" t="s">
         <v>18</v>
       </c>
       <c r="F81" s="2" t="s">
-        <v>488</v>
+        <v>486</v>
       </c>
       <c r="G81" s="2" t="s">
+        <v>487</v>
+      </c>
+      <c r="H81" s="2" t="s">
         <v>489</v>
-      </c>
-      <c r="H81" s="2" t="s">
-        <v>491</v>
       </c>
     </row>
     <row r="82" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
+        <v>499</v>
+      </c>
+      <c r="B82" t="s">
+        <v>490</v>
+      </c>
+      <c r="C82" s="2" t="s">
+        <v>500</v>
+      </c>
+      <c r="D82" s="2" t="s">
         <v>501</v>
-      </c>
-      <c r="B82" t="s">
-        <v>492</v>
-      </c>
-      <c r="C82" s="2" t="s">
-        <v>502</v>
-      </c>
-      <c r="D82" s="2" t="s">
-        <v>503</v>
       </c>
       <c r="E82" t="s">
         <v>146</v>
       </c>
       <c r="F82" s="2" t="s">
-        <v>499</v>
+        <v>497</v>
       </c>
       <c r="G82" s="2" t="s">
-        <v>499</v>
+        <v>497</v>
       </c>
       <c r="H82" s="2" t="s">
-        <v>500</v>
+        <v>498</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update REITs map data for 20260527
</commit_message>
<xml_diff>
--- a/REITs_location_updating.xlsx
+++ b/REITs_location_updating.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\21076\Desktop\公募REITs地图项目\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0C510B4E-6043-410C-94C5-55E5AFC44274}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{238E5B36-B7A9-4885-884A-21ABD847983C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="656" uniqueCount="504">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="664" uniqueCount="511">
   <si>
     <t>证券代码</t>
   </si>
@@ -1551,6 +1551,34 @@
   </si>
   <si>
     <t>{园博公寓，珩琦公寓，林边公寓，仁和公寓}</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>易方达广西北投高速公路</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>508093.SH</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>广西北部湾投资集团有限公司</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>南宁市</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>广西省</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>兰海高速广西南宁那南段</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>{兰海高速广西南宁那南段}</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
@@ -1621,12 +1649,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
@@ -1820,7 +1849,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H82"/>
+  <dimension ref="A1:H83"/>
   <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10.54296875" customWidth="1"/>
@@ -3963,6 +3992,32 @@
         <v>498</v>
       </c>
     </row>
+    <row r="83" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A83" s="2" t="s">
+        <v>505</v>
+      </c>
+      <c r="B83" s="2" t="s">
+        <v>504</v>
+      </c>
+      <c r="C83" s="2" t="s">
+        <v>506</v>
+      </c>
+      <c r="D83" s="2" t="s">
+        <v>509</v>
+      </c>
+      <c r="E83" t="s">
+        <v>18</v>
+      </c>
+      <c r="F83" s="2" t="s">
+        <v>507</v>
+      </c>
+      <c r="G83" s="3" t="s">
+        <v>508</v>
+      </c>
+      <c r="H83" s="3" t="s">
+        <v>510</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Refresh REITs map with standard Guangxi province name
</commit_message>
<xml_diff>
--- a/REITs_location_updating.xlsx
+++ b/REITs_location_updating.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\21076\Desktop\公募REITs地图项目\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{238E5B36-B7A9-4885-884A-21ABD847983C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4452590F-4E01-4344-B502-6D56F7E2611F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1570,15 +1570,15 @@
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
-    <t>广西省</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
     <t>兰海高速广西南宁那南段</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
     <t>{兰海高速广西南宁那南段}</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>广西壮族自治区</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
@@ -4003,7 +4003,7 @@
         <v>506</v>
       </c>
       <c r="D83" s="2" t="s">
-        <v>509</v>
+        <v>508</v>
       </c>
       <c r="E83" t="s">
         <v>18</v>
@@ -4011,11 +4011,11 @@
       <c r="F83" s="2" t="s">
         <v>507</v>
       </c>
-      <c r="G83" s="3" t="s">
-        <v>508</v>
+      <c r="G83" s="2" t="s">
+        <v>510</v>
       </c>
       <c r="H83" s="3" t="s">
-        <v>510</v>
+        <v>509</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Publish 20260728 REITs map update
</commit_message>
<xml_diff>
--- a/REITs_location_updating.xlsx
+++ b/REITs_location_updating.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\21076\Desktop\公募REITs地图项目\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{57A2FB3A-47C0-4661-B1F8-28ADE563C466}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A36BD83A-DA40-485A-A807-F7E72CCA7C77}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="已上市REITs" sheetId="1" r:id="rId1"/>
     <sheet name="未上市REITs" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="0" iterate="1" calcOnSave="0" concurrentManualCount="64"/>
   <extLst>
     <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
       <xlwcv:version setVersion="1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1096" uniqueCount="727">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1113" uniqueCount="742">
   <si>
     <t>证券代码</t>
   </si>
@@ -1303,9 +1303,6 @@
     <t>内蒙古自治区，内蒙古自治区</t>
   </si>
   <si>
-    <t>{华晨风电项目}|{恒润一期风电项目}</t>
-  </si>
-  <si>
     <t>180501.SZ</t>
   </si>
   <si>
@@ -1552,9 +1549,6 @@
     <t>南宁市</t>
   </si>
   <si>
-    <t>广西壮族自治区</t>
-  </si>
-  <si>
     <t>{兰海高速广西南宁那南段}</t>
   </si>
   <si>
@@ -1658,24 +1652,6 @@
   </si>
   <si>
     <t>{济南长清黄河公路大桥及其附属设施}</t>
-  </si>
-  <si>
-    <t>中航中核集团能源</t>
-  </si>
-  <si>
-    <t>中核汇能有限公司</t>
-  </si>
-  <si>
-    <t>新疆生产建设兵团第六师北塔山牧场境内的北塔山风电项目、广西壮族自治区贺州市富川瑶族自治县的富川协合风电项目</t>
-  </si>
-  <si>
-    <t>昌吉回族自治州，贺州市</t>
-  </si>
-  <si>
-    <t>新疆维吾尔自治区，广西壮族自治区</t>
-  </si>
-  <si>
-    <t>{北塔山风电项目}|{富川协合风电项目}</t>
   </si>
   <si>
     <t>山证晋中公投瑞阳供热</t>
@@ -2214,6 +2190,98 @@
   </si>
   <si>
     <t>华夏华润消费（扩募）</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>中航中核汇能新能源</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>508030.SH</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>中核汇能有限公司</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>北塔山风电项目、富川协合风电项目</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>新疆维吾尔自治区</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>广西壮族自治区</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>新疆维吾尔自治区，广西壮族自治区</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>{华晨风电项目}|{恒润一期风电项目}</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>{北塔山风电项目}|{富川协合风电项目}</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>昌吉回族自治洲，贺州市</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>东方红申能股份新能源</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>申能股份有限公司</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>乌兰20万千瓦风电项目</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>海西蒙古族藏族自治州‌</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>青海省</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>{乌兰20万千瓦风电项目}</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>南方润泽科技数据中心</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>基础设施REITs</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>河北省</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>廊坊市</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>润泽智算科技集团股份有限公司</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>{A-7数据中心，A-8数据中心 }</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve">A-7数据中心，A-8数据中心 </t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
@@ -2581,7 +2649,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I87"/>
+  <dimension ref="A1:I88"/>
   <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="2" width="12" customWidth="1"/>
@@ -4559,21 +4627,21 @@
         <v>424</v>
       </c>
       <c r="I68" t="s">
-        <v>425</v>
+        <v>726</v>
       </c>
     </row>
     <row r="69" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
+        <v>425</v>
+      </c>
+      <c r="B69" t="s">
         <v>426</v>
       </c>
-      <c r="B69" t="s">
+      <c r="C69" t="s">
         <v>427</v>
       </c>
-      <c r="C69" t="s">
+      <c r="D69" t="s">
         <v>428</v>
-      </c>
-      <c r="D69" t="s">
-        <v>429</v>
       </c>
       <c r="E69" t="s">
         <v>13</v>
@@ -4588,21 +4656,21 @@
         <v>337</v>
       </c>
       <c r="I69" t="s">
-        <v>430</v>
+        <v>429</v>
       </c>
     </row>
     <row r="70" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
+        <v>430</v>
+      </c>
+      <c r="B70" t="s">
         <v>431</v>
       </c>
-      <c r="B70" t="s">
+      <c r="C70" t="s">
         <v>432</v>
       </c>
-      <c r="C70" t="s">
+      <c r="D70" t="s">
         <v>433</v>
-      </c>
-      <c r="D70" t="s">
-        <v>434</v>
       </c>
       <c r="E70" t="s">
         <v>13</v>
@@ -4617,21 +4685,21 @@
         <v>337</v>
       </c>
       <c r="I70" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
     </row>
     <row r="71" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
+        <v>435</v>
+      </c>
+      <c r="B71" t="s">
+        <v>717</v>
+      </c>
+      <c r="C71" t="s">
         <v>436</v>
       </c>
-      <c r="B71" t="s">
-        <v>725</v>
-      </c>
-      <c r="C71" t="s">
+      <c r="D71" t="s">
         <v>437</v>
-      </c>
-      <c r="D71" t="s">
-        <v>438</v>
       </c>
       <c r="E71" t="s">
         <v>13</v>
@@ -4640,27 +4708,27 @@
         <v>29</v>
       </c>
       <c r="G71" t="s">
-        <v>439</v>
+        <v>438</v>
       </c>
       <c r="H71" t="s">
         <v>57</v>
       </c>
       <c r="I71" t="s">
-        <v>440</v>
+        <v>439</v>
       </c>
     </row>
     <row r="72" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
+        <v>440</v>
+      </c>
+      <c r="B72" t="s">
         <v>441</v>
       </c>
-      <c r="B72" t="s">
+      <c r="C72" t="s">
         <v>442</v>
       </c>
-      <c r="C72" t="s">
+      <c r="D72" t="s">
         <v>443</v>
-      </c>
-      <c r="D72" t="s">
-        <v>444</v>
       </c>
       <c r="E72" t="s">
         <v>13</v>
@@ -4675,21 +4743,21 @@
         <v>23</v>
       </c>
       <c r="I72" t="s">
-        <v>445</v>
+        <v>444</v>
       </c>
     </row>
     <row r="73" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
+        <v>445</v>
+      </c>
+      <c r="B73" t="s">
         <v>446</v>
       </c>
-      <c r="B73" t="s">
+      <c r="C73" t="s">
         <v>447</v>
       </c>
-      <c r="C73" t="s">
+      <c r="D73" t="s">
         <v>448</v>
-      </c>
-      <c r="D73" t="s">
-        <v>449</v>
       </c>
       <c r="E73" t="s">
         <v>13</v>
@@ -4704,21 +4772,21 @@
         <v>136</v>
       </c>
       <c r="I73" t="s">
-        <v>450</v>
+        <v>449</v>
       </c>
     </row>
     <row r="74" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
+        <v>450</v>
+      </c>
+      <c r="B74" t="s">
         <v>451</v>
       </c>
-      <c r="B74" t="s">
+      <c r="C74" t="s">
         <v>452</v>
       </c>
-      <c r="C74" t="s">
+      <c r="D74" t="s">
         <v>453</v>
-      </c>
-      <c r="D74" t="s">
-        <v>454</v>
       </c>
       <c r="E74" t="s">
         <v>13</v>
@@ -4727,27 +4795,27 @@
         <v>29</v>
       </c>
       <c r="G74" t="s">
-        <v>455</v>
+        <v>454</v>
       </c>
       <c r="H74" t="s">
         <v>206</v>
       </c>
       <c r="I74" t="s">
-        <v>456</v>
+        <v>455</v>
       </c>
     </row>
     <row r="75" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
+        <v>456</v>
+      </c>
+      <c r="B75" t="s">
         <v>457</v>
       </c>
-      <c r="B75" t="s">
+      <c r="C75" t="s">
         <v>458</v>
       </c>
-      <c r="C75" t="s">
+      <c r="D75" t="s">
         <v>459</v>
-      </c>
-      <c r="D75" t="s">
-        <v>460</v>
       </c>
       <c r="E75" t="s">
         <v>13</v>
@@ -4762,21 +4830,21 @@
         <v>57</v>
       </c>
       <c r="I75" t="s">
-        <v>461</v>
+        <v>460</v>
       </c>
     </row>
     <row r="76" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
+        <v>461</v>
+      </c>
+      <c r="B76" t="s">
         <v>462</v>
       </c>
-      <c r="B76" t="s">
+      <c r="C76" t="s">
         <v>463</v>
       </c>
-      <c r="C76" t="s">
+      <c r="D76" t="s">
         <v>464</v>
-      </c>
-      <c r="D76" t="s">
-        <v>465</v>
       </c>
       <c r="E76" t="s">
         <v>13</v>
@@ -4785,56 +4853,56 @@
         <v>29</v>
       </c>
       <c r="G76" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
       <c r="H76" t="s">
         <v>337</v>
       </c>
       <c r="I76" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
     </row>
     <row r="77" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
+        <v>467</v>
+      </c>
+      <c r="B77" t="s">
         <v>468</v>
       </c>
-      <c r="B77" t="s">
+      <c r="C77" t="s">
         <v>469</v>
       </c>
-      <c r="C77" t="s">
+      <c r="D77" t="s">
         <v>470</v>
       </c>
-      <c r="D77" t="s">
+      <c r="E77" t="s">
+        <v>13</v>
+      </c>
+      <c r="F77" t="s">
         <v>471</v>
       </c>
-      <c r="E77" t="s">
-        <v>13</v>
-      </c>
-      <c r="F77" t="s">
+      <c r="G77" t="s">
         <v>472</v>
-      </c>
-      <c r="G77" t="s">
-        <v>473</v>
       </c>
       <c r="H77" t="s">
         <v>23</v>
       </c>
       <c r="I77" t="s">
-        <v>474</v>
+        <v>473</v>
       </c>
     </row>
     <row r="78" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
+        <v>474</v>
+      </c>
+      <c r="B78" t="s">
         <v>475</v>
       </c>
-      <c r="B78" t="s">
+      <c r="C78" t="s">
         <v>476</v>
       </c>
-      <c r="C78" t="s">
+      <c r="D78" t="s">
         <v>477</v>
-      </c>
-      <c r="D78" t="s">
-        <v>478</v>
       </c>
       <c r="E78" t="s">
         <v>13</v>
@@ -4849,21 +4917,21 @@
         <v>35</v>
       </c>
       <c r="I78" t="s">
-        <v>479</v>
+        <v>478</v>
       </c>
     </row>
     <row r="79" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
+        <v>479</v>
+      </c>
+      <c r="B79" t="s">
         <v>480</v>
       </c>
-      <c r="B79" t="s">
+      <c r="C79" t="s">
         <v>481</v>
       </c>
-      <c r="C79" t="s">
+      <c r="D79" t="s">
         <v>482</v>
-      </c>
-      <c r="D79" t="s">
-        <v>483</v>
       </c>
       <c r="E79" t="s">
         <v>13</v>
@@ -4872,27 +4940,27 @@
         <v>212</v>
       </c>
       <c r="G79" t="s">
-        <v>484</v>
+        <v>483</v>
       </c>
       <c r="H79" t="s">
         <v>266</v>
       </c>
       <c r="I79" t="s">
-        <v>485</v>
+        <v>484</v>
       </c>
     </row>
     <row r="80" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
+        <v>485</v>
+      </c>
+      <c r="B80" t="s">
         <v>486</v>
       </c>
-      <c r="B80" t="s">
+      <c r="C80" t="s">
         <v>487</v>
       </c>
-      <c r="C80" t="s">
+      <c r="D80" t="s">
         <v>488</v>
-      </c>
-      <c r="D80" t="s">
-        <v>489</v>
       </c>
       <c r="E80" t="s">
         <v>13</v>
@@ -4901,27 +4969,27 @@
         <v>91</v>
       </c>
       <c r="G80" t="s">
+        <v>489</v>
+      </c>
+      <c r="H80" t="s">
+        <v>723</v>
+      </c>
+      <c r="I80" t="s">
         <v>490</v>
-      </c>
-      <c r="H80" t="s">
-        <v>287</v>
-      </c>
-      <c r="I80" t="s">
-        <v>491</v>
       </c>
     </row>
     <row r="81" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
+        <v>491</v>
+      </c>
+      <c r="B81" t="s">
         <v>492</v>
       </c>
-      <c r="B81" t="s">
+      <c r="C81" t="s">
         <v>493</v>
       </c>
-      <c r="C81" t="s">
+      <c r="D81" t="s">
         <v>494</v>
-      </c>
-      <c r="D81" t="s">
-        <v>495</v>
       </c>
       <c r="E81" t="s">
         <v>13</v>
@@ -4930,27 +4998,27 @@
         <v>21</v>
       </c>
       <c r="G81" t="s">
-        <v>496</v>
+        <v>495</v>
       </c>
       <c r="H81" t="s">
         <v>176</v>
       </c>
       <c r="I81" t="s">
-        <v>497</v>
+        <v>496</v>
       </c>
     </row>
     <row r="82" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
+        <v>497</v>
+      </c>
+      <c r="B82" t="s">
         <v>498</v>
       </c>
-      <c r="B82" t="s">
+      <c r="C82" t="s">
         <v>499</v>
       </c>
-      <c r="C82" t="s">
+      <c r="D82" t="s">
         <v>500</v>
-      </c>
-      <c r="D82" t="s">
-        <v>501</v>
       </c>
       <c r="E82" t="s">
         <v>13</v>
@@ -4965,21 +5033,21 @@
         <v>35</v>
       </c>
       <c r="I82" t="s">
-        <v>502</v>
+        <v>501</v>
       </c>
     </row>
     <row r="83" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
+        <v>502</v>
+      </c>
+      <c r="B83" t="s">
         <v>503</v>
       </c>
-      <c r="B83" t="s">
+      <c r="C83" t="s">
         <v>504</v>
       </c>
-      <c r="C83" t="s">
+      <c r="D83" t="s">
         <v>505</v>
-      </c>
-      <c r="D83" t="s">
-        <v>506</v>
       </c>
       <c r="E83" t="s">
         <v>13</v>
@@ -4988,91 +5056,91 @@
         <v>21</v>
       </c>
       <c r="G83" t="s">
+        <v>506</v>
+      </c>
+      <c r="H83" t="s">
+        <v>724</v>
+      </c>
+      <c r="I83" t="s">
         <v>507</v>
-      </c>
-      <c r="H83" t="s">
-        <v>508</v>
-      </c>
-      <c r="I83" t="s">
-        <v>509</v>
       </c>
     </row>
     <row r="84" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
+        <v>508</v>
+      </c>
+      <c r="B84" t="s">
+        <v>509</v>
+      </c>
+      <c r="C84" t="s">
         <v>510</v>
       </c>
-      <c r="B84" t="s">
+      <c r="D84" t="s">
         <v>511</v>
       </c>
-      <c r="C84" t="s">
+      <c r="E84" t="s">
         <v>512</v>
       </c>
-      <c r="D84" t="s">
+      <c r="F84" t="s">
         <v>513</v>
       </c>
-      <c r="E84" t="s">
+      <c r="G84" t="s">
         <v>514</v>
       </c>
-      <c r="F84" t="s">
+      <c r="H84" t="s">
         <v>515</v>
       </c>
-      <c r="G84" t="s">
+      <c r="I84" t="s">
         <v>516</v>
-      </c>
-      <c r="H84" t="s">
-        <v>517</v>
-      </c>
-      <c r="I84" t="s">
-        <v>518</v>
       </c>
     </row>
     <row r="85" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
-        <v>519</v>
+        <v>517</v>
       </c>
       <c r="B85" t="s">
-        <v>520</v>
+        <v>518</v>
       </c>
       <c r="C85" t="s">
         <v>247</v>
       </c>
       <c r="D85" t="s">
+        <v>519</v>
+      </c>
+      <c r="E85" t="s">
+        <v>512</v>
+      </c>
+      <c r="F85" t="s">
+        <v>513</v>
+      </c>
+      <c r="G85" t="s">
+        <v>520</v>
+      </c>
+      <c r="H85" t="s">
         <v>521</v>
       </c>
-      <c r="E85" t="s">
-        <v>514</v>
-      </c>
-      <c r="F85" t="s">
-        <v>515</v>
-      </c>
-      <c r="G85" t="s">
+      <c r="I85" t="s">
         <v>522</v>
-      </c>
-      <c r="H85" t="s">
-        <v>523</v>
-      </c>
-      <c r="I85" t="s">
-        <v>524</v>
       </c>
     </row>
     <row r="86" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
+        <v>523</v>
+      </c>
+      <c r="B86" t="s">
+        <v>524</v>
+      </c>
+      <c r="C86" t="s">
         <v>525</v>
       </c>
-      <c r="B86" t="s">
+      <c r="D86" t="s">
         <v>526</v>
       </c>
-      <c r="C86" t="s">
+      <c r="E86" t="s">
+        <v>512</v>
+      </c>
+      <c r="F86" t="s">
         <v>527</v>
-      </c>
-      <c r="D86" t="s">
-        <v>528</v>
-      </c>
-      <c r="E86" t="s">
-        <v>514</v>
-      </c>
-      <c r="F86" t="s">
-        <v>529</v>
       </c>
       <c r="G86" t="s">
         <v>35</v>
@@ -5081,27 +5149,27 @@
         <v>35</v>
       </c>
       <c r="I86" t="s">
-        <v>530</v>
+        <v>528</v>
       </c>
     </row>
     <row r="87" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
-        <v>719</v>
+        <v>711</v>
       </c>
       <c r="B87" t="s">
+        <v>529</v>
+      </c>
+      <c r="C87" t="s">
+        <v>530</v>
+      </c>
+      <c r="D87" t="s">
+        <v>712</v>
+      </c>
+      <c r="E87" t="s">
+        <v>512</v>
+      </c>
+      <c r="F87" t="s">
         <v>531</v>
-      </c>
-      <c r="C87" t="s">
-        <v>532</v>
-      </c>
-      <c r="D87" t="s">
-        <v>720</v>
-      </c>
-      <c r="E87" t="s">
-        <v>514</v>
-      </c>
-      <c r="F87" t="s">
-        <v>533</v>
       </c>
       <c r="G87" t="s">
         <v>15</v>
@@ -5110,7 +5178,36 @@
         <v>15</v>
       </c>
       <c r="I87" t="s">
-        <v>534</v>
+        <v>532</v>
+      </c>
+    </row>
+    <row r="88" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A88" t="s">
+        <v>720</v>
+      </c>
+      <c r="B88" t="s">
+        <v>719</v>
+      </c>
+      <c r="C88" t="s">
+        <v>721</v>
+      </c>
+      <c r="D88" t="s">
+        <v>722</v>
+      </c>
+      <c r="E88" t="s">
+        <v>13</v>
+      </c>
+      <c r="F88" t="s">
+        <v>91</v>
+      </c>
+      <c r="G88" t="s">
+        <v>728</v>
+      </c>
+      <c r="H88" t="s">
+        <v>725</v>
+      </c>
+      <c r="I88" t="s">
+        <v>727</v>
       </c>
     </row>
   </sheetData>
@@ -5121,7 +5218,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:I39"/>
+  <dimension ref="A1:I40"/>
   <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -5166,13 +5263,13 @@
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="B2" t="s">
+        <v>533</v>
+      </c>
+      <c r="C2" t="s">
+        <v>534</v>
+      </c>
+      <c r="D2" t="s">
         <v>535</v>
-      </c>
-      <c r="C2" t="s">
-        <v>536</v>
-      </c>
-      <c r="D2" t="s">
-        <v>537</v>
       </c>
       <c r="E2" t="s">
         <v>13</v>
@@ -5181,24 +5278,24 @@
         <v>91</v>
       </c>
       <c r="G2" t="s">
-        <v>538</v>
+        <v>536</v>
       </c>
       <c r="H2" t="s">
         <v>156</v>
       </c>
       <c r="I2" t="s">
-        <v>539</v>
+        <v>537</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="B3" t="s">
+        <v>538</v>
+      </c>
+      <c r="C3" t="s">
+        <v>539</v>
+      </c>
+      <c r="D3" t="s">
         <v>540</v>
-      </c>
-      <c r="C3" t="s">
-        <v>541</v>
-      </c>
-      <c r="D3" t="s">
-        <v>542</v>
       </c>
       <c r="E3" t="s">
         <v>13</v>
@@ -5213,96 +5310,96 @@
         <v>57</v>
       </c>
       <c r="I3" t="s">
-        <v>543</v>
+        <v>541</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="B4" t="s">
+        <v>542</v>
+      </c>
+      <c r="C4" t="s">
+        <v>543</v>
+      </c>
+      <c r="D4" t="s">
         <v>544</v>
       </c>
-      <c r="C4" t="s">
+      <c r="E4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F4" t="s">
+        <v>272</v>
+      </c>
+      <c r="G4" t="s">
         <v>545</v>
       </c>
-      <c r="D4" t="s">
+      <c r="H4" t="s">
         <v>546</v>
       </c>
-      <c r="E4" t="s">
-        <v>13</v>
-      </c>
-      <c r="F4" t="s">
-        <v>91</v>
-      </c>
-      <c r="G4" t="s">
+      <c r="I4" t="s">
         <v>547</v>
-      </c>
-      <c r="H4" t="s">
-        <v>548</v>
-      </c>
-      <c r="I4" t="s">
-        <v>549</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="B5" t="s">
+        <v>548</v>
+      </c>
+      <c r="C5" t="s">
+        <v>549</v>
+      </c>
+      <c r="D5" t="s">
         <v>550</v>
       </c>
-      <c r="C5" t="s">
+      <c r="E5" t="s">
+        <v>13</v>
+      </c>
+      <c r="F5" t="s">
+        <v>21</v>
+      </c>
+      <c r="G5" t="s">
         <v>551</v>
       </c>
-      <c r="D5" t="s">
+      <c r="H5" t="s">
+        <v>112</v>
+      </c>
+      <c r="I5" t="s">
         <v>552</v>
-      </c>
-      <c r="E5" t="s">
-        <v>13</v>
-      </c>
-      <c r="F5" t="s">
-        <v>272</v>
-      </c>
-      <c r="G5" t="s">
-        <v>553</v>
-      </c>
-      <c r="H5" t="s">
-        <v>554</v>
-      </c>
-      <c r="I5" t="s">
-        <v>555</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="B6" t="s">
+        <v>553</v>
+      </c>
+      <c r="C6" t="s">
+        <v>554</v>
+      </c>
+      <c r="D6" t="s">
+        <v>555</v>
+      </c>
+      <c r="E6" t="s">
+        <v>13</v>
+      </c>
+      <c r="F6" t="s">
+        <v>14</v>
+      </c>
+      <c r="G6" t="s">
+        <v>514</v>
+      </c>
+      <c r="H6" t="s">
+        <v>515</v>
+      </c>
+      <c r="I6" t="s">
         <v>556</v>
-      </c>
-      <c r="C6" t="s">
-        <v>557</v>
-      </c>
-      <c r="D6" t="s">
-        <v>558</v>
-      </c>
-      <c r="E6" t="s">
-        <v>13</v>
-      </c>
-      <c r="F6" t="s">
-        <v>21</v>
-      </c>
-      <c r="G6" t="s">
-        <v>559</v>
-      </c>
-      <c r="H6" t="s">
-        <v>112</v>
-      </c>
-      <c r="I6" t="s">
-        <v>560</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="B7" t="s">
-        <v>561</v>
+        <v>557</v>
       </c>
       <c r="C7" t="s">
-        <v>562</v>
+        <v>558</v>
       </c>
       <c r="D7" t="s">
-        <v>563</v>
+        <v>559</v>
       </c>
       <c r="E7" t="s">
         <v>13</v>
@@ -5311,648 +5408,648 @@
         <v>14</v>
       </c>
       <c r="G7" t="s">
-        <v>516</v>
+        <v>205</v>
       </c>
       <c r="H7" t="s">
-        <v>517</v>
+        <v>206</v>
       </c>
       <c r="I7" t="s">
-        <v>564</v>
+        <v>560</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="B8" t="s">
-        <v>565</v>
+        <v>718</v>
       </c>
       <c r="C8" t="s">
-        <v>566</v>
+        <v>436</v>
       </c>
       <c r="D8" t="s">
-        <v>567</v>
+        <v>561</v>
       </c>
       <c r="E8" t="s">
         <v>13</v>
       </c>
       <c r="F8" t="s">
-        <v>14</v>
+        <v>29</v>
       </c>
       <c r="G8" t="s">
-        <v>205</v>
+        <v>142</v>
       </c>
       <c r="H8" t="s">
-        <v>206</v>
+        <v>143</v>
       </c>
       <c r="I8" t="s">
-        <v>568</v>
+        <v>562</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="B9" t="s">
-        <v>726</v>
+        <v>563</v>
       </c>
       <c r="C9" t="s">
-        <v>437</v>
+        <v>564</v>
       </c>
       <c r="D9" t="s">
-        <v>569</v>
+        <v>565</v>
       </c>
       <c r="E9" t="s">
-        <v>13</v>
+        <v>512</v>
       </c>
       <c r="F9" t="s">
-        <v>29</v>
+        <v>566</v>
       </c>
       <c r="G9" t="s">
-        <v>142</v>
+        <v>567</v>
       </c>
       <c r="H9" t="s">
-        <v>143</v>
+        <v>568</v>
       </c>
       <c r="I9" t="s">
-        <v>570</v>
+        <v>713</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="B10" t="s">
+        <v>569</v>
+      </c>
+      <c r="C10" t="s">
+        <v>570</v>
+      </c>
+      <c r="D10" t="s">
         <v>571</v>
       </c>
-      <c r="C10" t="s">
+      <c r="E10" t="s">
+        <v>512</v>
+      </c>
+      <c r="F10" t="s">
         <v>572</v>
       </c>
-      <c r="D10" t="s">
+      <c r="G10" t="s">
+        <v>15</v>
+      </c>
+      <c r="H10" t="s">
+        <v>15</v>
+      </c>
+      <c r="I10" t="s">
         <v>573</v>
-      </c>
-      <c r="E10" t="s">
-        <v>514</v>
-      </c>
-      <c r="F10" t="s">
-        <v>574</v>
-      </c>
-      <c r="G10" t="s">
-        <v>575</v>
-      </c>
-      <c r="H10" t="s">
-        <v>576</v>
-      </c>
-      <c r="I10" t="s">
-        <v>721</v>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="B11" t="s">
+        <v>574</v>
+      </c>
+      <c r="C11" t="s">
+        <v>575</v>
+      </c>
+      <c r="D11" t="s">
+        <v>576</v>
+      </c>
+      <c r="E11" t="s">
+        <v>512</v>
+      </c>
+      <c r="F11" t="s">
         <v>577</v>
       </c>
-      <c r="C11" t="s">
+      <c r="G11" t="s">
         <v>578</v>
       </c>
-      <c r="D11" t="s">
+      <c r="H11" t="s">
         <v>579</v>
       </c>
-      <c r="E11" t="s">
-        <v>514</v>
-      </c>
-      <c r="F11" t="s">
+      <c r="I11" t="s">
         <v>580</v>
-      </c>
-      <c r="G11" t="s">
-        <v>15</v>
-      </c>
-      <c r="H11" t="s">
-        <v>15</v>
-      </c>
-      <c r="I11" t="s">
-        <v>581</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="B12" t="s">
+        <v>581</v>
+      </c>
+      <c r="C12" t="s">
         <v>582</v>
       </c>
-      <c r="C12" t="s">
+      <c r="D12" t="s">
         <v>583</v>
       </c>
-      <c r="D12" t="s">
+      <c r="E12" t="s">
+        <v>512</v>
+      </c>
+      <c r="F12" t="s">
+        <v>527</v>
+      </c>
+      <c r="G12" t="s">
+        <v>343</v>
+      </c>
+      <c r="H12" t="s">
+        <v>344</v>
+      </c>
+      <c r="I12" t="s">
         <v>584</v>
-      </c>
-      <c r="E12" t="s">
-        <v>514</v>
-      </c>
-      <c r="F12" t="s">
-        <v>585</v>
-      </c>
-      <c r="G12" t="s">
-        <v>586</v>
-      </c>
-      <c r="H12" t="s">
-        <v>587</v>
-      </c>
-      <c r="I12" t="s">
-        <v>588</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="B13" t="s">
+        <v>585</v>
+      </c>
+      <c r="C13" t="s">
+        <v>586</v>
+      </c>
+      <c r="D13" t="s">
+        <v>587</v>
+      </c>
+      <c r="E13" t="s">
+        <v>512</v>
+      </c>
+      <c r="F13" t="s">
+        <v>572</v>
+      </c>
+      <c r="G13" t="s">
+        <v>588</v>
+      </c>
+      <c r="H13" t="s">
+        <v>412</v>
+      </c>
+      <c r="I13" t="s">
         <v>589</v>
-      </c>
-      <c r="C13" t="s">
-        <v>590</v>
-      </c>
-      <c r="D13" t="s">
-        <v>591</v>
-      </c>
-      <c r="E13" t="s">
-        <v>514</v>
-      </c>
-      <c r="F13" t="s">
-        <v>529</v>
-      </c>
-      <c r="G13" t="s">
-        <v>343</v>
-      </c>
-      <c r="H13" t="s">
-        <v>344</v>
-      </c>
-      <c r="I13" t="s">
-        <v>592</v>
       </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.25">
       <c r="B14" t="s">
+        <v>590</v>
+      </c>
+      <c r="C14" t="s">
+        <v>591</v>
+      </c>
+      <c r="D14" t="s">
+        <v>592</v>
+      </c>
+      <c r="E14" t="s">
+        <v>512</v>
+      </c>
+      <c r="F14" t="s">
+        <v>566</v>
+      </c>
+      <c r="G14" t="s">
         <v>593</v>
       </c>
-      <c r="C14" t="s">
+      <c r="H14" t="s">
         <v>594</v>
       </c>
-      <c r="D14" t="s">
+      <c r="I14" t="s">
         <v>595</v>
-      </c>
-      <c r="E14" t="s">
-        <v>514</v>
-      </c>
-      <c r="F14" t="s">
-        <v>580</v>
-      </c>
-      <c r="G14" t="s">
-        <v>596</v>
-      </c>
-      <c r="H14" t="s">
-        <v>412</v>
-      </c>
-      <c r="I14" t="s">
-        <v>597</v>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.25">
       <c r="B15" t="s">
+        <v>596</v>
+      </c>
+      <c r="C15" t="s">
+        <v>597</v>
+      </c>
+      <c r="D15" t="s">
         <v>598</v>
       </c>
-      <c r="C15" t="s">
+      <c r="E15" t="s">
+        <v>512</v>
+      </c>
+      <c r="F15" t="s">
+        <v>527</v>
+      </c>
+      <c r="G15" t="s">
         <v>599</v>
       </c>
-      <c r="D15" t="s">
+      <c r="H15" t="s">
         <v>600</v>
       </c>
-      <c r="E15" t="s">
-        <v>514</v>
-      </c>
-      <c r="F15" t="s">
-        <v>574</v>
-      </c>
-      <c r="G15" t="s">
+      <c r="I15" t="s">
         <v>601</v>
-      </c>
-      <c r="H15" t="s">
-        <v>602</v>
-      </c>
-      <c r="I15" t="s">
-        <v>603</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.25">
       <c r="B16" t="s">
+        <v>602</v>
+      </c>
+      <c r="C16" t="s">
+        <v>603</v>
+      </c>
+      <c r="D16" t="s">
         <v>604</v>
       </c>
-      <c r="C16" t="s">
+      <c r="E16" t="s">
+        <v>512</v>
+      </c>
+      <c r="F16" t="s">
+        <v>527</v>
+      </c>
+      <c r="G16" t="s">
+        <v>15</v>
+      </c>
+      <c r="H16" t="s">
+        <v>15</v>
+      </c>
+      <c r="I16" t="s">
         <v>605</v>
-      </c>
-      <c r="D16" t="s">
-        <v>606</v>
-      </c>
-      <c r="E16" t="s">
-        <v>514</v>
-      </c>
-      <c r="F16" t="s">
-        <v>529</v>
-      </c>
-      <c r="G16" t="s">
-        <v>607</v>
-      </c>
-      <c r="H16" t="s">
-        <v>608</v>
-      </c>
-      <c r="I16" t="s">
-        <v>609</v>
       </c>
     </row>
     <row r="17" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B17" t="s">
+        <v>606</v>
+      </c>
+      <c r="C17" t="s">
+        <v>607</v>
+      </c>
+      <c r="D17" t="s">
+        <v>608</v>
+      </c>
+      <c r="E17" t="s">
+        <v>13</v>
+      </c>
+      <c r="F17" t="s">
+        <v>609</v>
+      </c>
+      <c r="G17" t="s">
+        <v>129</v>
+      </c>
+      <c r="H17" t="s">
+        <v>129</v>
+      </c>
+      <c r="I17" t="s">
         <v>610</v>
-      </c>
-      <c r="C17" t="s">
-        <v>611</v>
-      </c>
-      <c r="D17" t="s">
-        <v>612</v>
-      </c>
-      <c r="E17" t="s">
-        <v>514</v>
-      </c>
-      <c r="F17" t="s">
-        <v>529</v>
-      </c>
-      <c r="G17" t="s">
-        <v>15</v>
-      </c>
-      <c r="H17" t="s">
-        <v>15</v>
-      </c>
-      <c r="I17" t="s">
-        <v>613</v>
       </c>
     </row>
     <row r="18" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B18" t="s">
+        <v>611</v>
+      </c>
+      <c r="C18" t="s">
+        <v>612</v>
+      </c>
+      <c r="D18" t="s">
+        <v>613</v>
+      </c>
+      <c r="E18" t="s">
+        <v>13</v>
+      </c>
+      <c r="F18" t="s">
+        <v>91</v>
+      </c>
+      <c r="G18" t="s">
         <v>614</v>
       </c>
-      <c r="C18" t="s">
+      <c r="H18" t="s">
         <v>615</v>
       </c>
-      <c r="D18" t="s">
+      <c r="I18" t="s">
         <v>616</v>
-      </c>
-      <c r="E18" t="s">
-        <v>13</v>
-      </c>
-      <c r="F18" t="s">
-        <v>617</v>
-      </c>
-      <c r="G18" t="s">
-        <v>129</v>
-      </c>
-      <c r="H18" t="s">
-        <v>129</v>
-      </c>
-      <c r="I18" t="s">
-        <v>618</v>
       </c>
     </row>
     <row r="19" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B19" t="s">
+        <v>617</v>
+      </c>
+      <c r="C19" t="s">
+        <v>618</v>
+      </c>
+      <c r="D19" t="s">
         <v>619</v>
       </c>
-      <c r="C19" t="s">
+      <c r="E19" t="s">
+        <v>512</v>
+      </c>
+      <c r="F19" t="s">
+        <v>527</v>
+      </c>
+      <c r="G19" t="s">
+        <v>35</v>
+      </c>
+      <c r="H19" t="s">
+        <v>35</v>
+      </c>
+      <c r="I19" t="s">
         <v>620</v>
-      </c>
-      <c r="D19" t="s">
-        <v>621</v>
-      </c>
-      <c r="E19" t="s">
-        <v>13</v>
-      </c>
-      <c r="F19" t="s">
-        <v>91</v>
-      </c>
-      <c r="G19" t="s">
-        <v>622</v>
-      </c>
-      <c r="H19" t="s">
-        <v>623</v>
-      </c>
-      <c r="I19" t="s">
-        <v>624</v>
       </c>
     </row>
     <row r="20" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B20" t="s">
+        <v>621</v>
+      </c>
+      <c r="C20" t="s">
+        <v>622</v>
+      </c>
+      <c r="D20" t="s">
+        <v>623</v>
+      </c>
+      <c r="E20" t="s">
+        <v>512</v>
+      </c>
+      <c r="F20" t="s">
+        <v>527</v>
+      </c>
+      <c r="G20" t="s">
+        <v>624</v>
+      </c>
+      <c r="H20" t="s">
         <v>625</v>
       </c>
-      <c r="C20" t="s">
+      <c r="I20" t="s">
         <v>626</v>
-      </c>
-      <c r="D20" t="s">
-        <v>627</v>
-      </c>
-      <c r="E20" t="s">
-        <v>514</v>
-      </c>
-      <c r="F20" t="s">
-        <v>529</v>
-      </c>
-      <c r="G20" t="s">
-        <v>35</v>
-      </c>
-      <c r="H20" t="s">
-        <v>35</v>
-      </c>
-      <c r="I20" t="s">
-        <v>628</v>
       </c>
     </row>
     <row r="21" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B21" t="s">
+        <v>627</v>
+      </c>
+      <c r="C21" t="s">
+        <v>628</v>
+      </c>
+      <c r="D21" t="s">
         <v>629</v>
       </c>
-      <c r="C21" t="s">
+      <c r="E21" t="s">
+        <v>512</v>
+      </c>
+      <c r="F21" t="s">
+        <v>527</v>
+      </c>
+      <c r="G21" t="s">
+        <v>336</v>
+      </c>
+      <c r="H21" t="s">
+        <v>337</v>
+      </c>
+      <c r="I21" t="s">
         <v>630</v>
-      </c>
-      <c r="D21" t="s">
-        <v>631</v>
-      </c>
-      <c r="E21" t="s">
-        <v>514</v>
-      </c>
-      <c r="F21" t="s">
-        <v>529</v>
-      </c>
-      <c r="G21" t="s">
-        <v>632</v>
-      </c>
-      <c r="H21" t="s">
-        <v>633</v>
-      </c>
-      <c r="I21" t="s">
-        <v>634</v>
       </c>
     </row>
     <row r="22" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B22" t="s">
+        <v>631</v>
+      </c>
+      <c r="C22" t="s">
+        <v>632</v>
+      </c>
+      <c r="D22" t="s">
+        <v>633</v>
+      </c>
+      <c r="E22" t="s">
+        <v>512</v>
+      </c>
+      <c r="F22" t="s">
+        <v>634</v>
+      </c>
+      <c r="G22" t="s">
         <v>635</v>
       </c>
-      <c r="C22" t="s">
+      <c r="H22" t="s">
         <v>636</v>
       </c>
-      <c r="D22" t="s">
+      <c r="I22" t="s">
         <v>637</v>
-      </c>
-      <c r="E22" t="s">
-        <v>514</v>
-      </c>
-      <c r="F22" t="s">
-        <v>529</v>
-      </c>
-      <c r="G22" t="s">
-        <v>336</v>
-      </c>
-      <c r="H22" t="s">
-        <v>337</v>
-      </c>
-      <c r="I22" t="s">
-        <v>638</v>
       </c>
     </row>
     <row r="23" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B23" t="s">
+        <v>638</v>
+      </c>
+      <c r="C23" t="s">
         <v>639</v>
       </c>
-      <c r="C23" t="s">
+      <c r="D23" t="s">
         <v>640</v>
       </c>
-      <c r="D23" t="s">
+      <c r="E23" t="s">
+        <v>512</v>
+      </c>
+      <c r="F23" t="s">
+        <v>572</v>
+      </c>
+      <c r="G23" t="s">
+        <v>35</v>
+      </c>
+      <c r="H23" t="s">
+        <v>35</v>
+      </c>
+      <c r="I23" t="s">
         <v>641</v>
-      </c>
-      <c r="E23" t="s">
-        <v>514</v>
-      </c>
-      <c r="F23" t="s">
-        <v>642</v>
-      </c>
-      <c r="G23" t="s">
-        <v>643</v>
-      </c>
-      <c r="H23" t="s">
-        <v>644</v>
-      </c>
-      <c r="I23" t="s">
-        <v>645</v>
       </c>
     </row>
     <row r="24" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B24" t="s">
-        <v>646</v>
+        <v>642</v>
       </c>
       <c r="C24" t="s">
-        <v>647</v>
+        <v>643</v>
       </c>
       <c r="D24" t="s">
-        <v>648</v>
+        <v>644</v>
       </c>
       <c r="E24" t="s">
-        <v>514</v>
+        <v>13</v>
       </c>
       <c r="F24" t="s">
-        <v>580</v>
+        <v>162</v>
       </c>
       <c r="G24" t="s">
-        <v>35</v>
+        <v>15</v>
       </c>
       <c r="H24" t="s">
-        <v>35</v>
+        <v>15</v>
       </c>
       <c r="I24" t="s">
-        <v>649</v>
+        <v>645</v>
       </c>
     </row>
     <row r="25" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B25" t="s">
+        <v>646</v>
+      </c>
+      <c r="C25" t="s">
+        <v>647</v>
+      </c>
+      <c r="D25" t="s">
+        <v>648</v>
+      </c>
+      <c r="E25" t="s">
+        <v>13</v>
+      </c>
+      <c r="F25" t="s">
+        <v>471</v>
+      </c>
+      <c r="G25" t="s">
+        <v>649</v>
+      </c>
+      <c r="H25" t="s">
+        <v>412</v>
+      </c>
+      <c r="I25" t="s">
         <v>650</v>
-      </c>
-      <c r="C25" t="s">
-        <v>651</v>
-      </c>
-      <c r="D25" t="s">
-        <v>652</v>
-      </c>
-      <c r="E25" t="s">
-        <v>13</v>
-      </c>
-      <c r="F25" t="s">
-        <v>162</v>
-      </c>
-      <c r="G25" t="s">
-        <v>15</v>
-      </c>
-      <c r="H25" t="s">
-        <v>15</v>
-      </c>
-      <c r="I25" t="s">
-        <v>653</v>
       </c>
     </row>
     <row r="26" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B26" t="s">
+        <v>651</v>
+      </c>
+      <c r="C26" t="s">
+        <v>652</v>
+      </c>
+      <c r="D26" t="s">
+        <v>653</v>
+      </c>
+      <c r="E26" t="s">
+        <v>13</v>
+      </c>
+      <c r="F26" t="s">
+        <v>187</v>
+      </c>
+      <c r="G26" t="s">
         <v>654</v>
       </c>
-      <c r="C26" t="s">
+      <c r="H26" t="s">
+        <v>23</v>
+      </c>
+      <c r="I26" t="s">
         <v>655</v>
-      </c>
-      <c r="D26" t="s">
-        <v>656</v>
-      </c>
-      <c r="E26" t="s">
-        <v>13</v>
-      </c>
-      <c r="F26" t="s">
-        <v>472</v>
-      </c>
-      <c r="G26" t="s">
-        <v>657</v>
-      </c>
-      <c r="H26" t="s">
-        <v>412</v>
-      </c>
-      <c r="I26" t="s">
-        <v>658</v>
       </c>
     </row>
     <row r="27" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B27" t="s">
+        <v>656</v>
+      </c>
+      <c r="C27" t="s">
+        <v>657</v>
+      </c>
+      <c r="D27" t="s">
+        <v>658</v>
+      </c>
+      <c r="E27" t="s">
+        <v>512</v>
+      </c>
+      <c r="F27" t="s">
+        <v>566</v>
+      </c>
+      <c r="G27" t="s">
         <v>659</v>
       </c>
-      <c r="C27" t="s">
+      <c r="H27" t="s">
         <v>660</v>
       </c>
-      <c r="D27" t="s">
+      <c r="I27" t="s">
         <v>661</v>
-      </c>
-      <c r="E27" t="s">
-        <v>13</v>
-      </c>
-      <c r="F27" t="s">
-        <v>187</v>
-      </c>
-      <c r="G27" t="s">
-        <v>662</v>
-      </c>
-      <c r="H27" t="s">
-        <v>23</v>
-      </c>
-      <c r="I27" t="s">
-        <v>663</v>
       </c>
     </row>
     <row r="28" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B28" t="s">
+        <v>716</v>
+      </c>
+      <c r="C28" t="s">
+        <v>662</v>
+      </c>
+      <c r="D28" t="s">
+        <v>663</v>
+      </c>
+      <c r="E28" t="s">
+        <v>512</v>
+      </c>
+      <c r="F28" t="s">
+        <v>527</v>
+      </c>
+      <c r="G28" t="s">
         <v>664</v>
       </c>
-      <c r="C28" t="s">
+      <c r="H28" t="s">
         <v>665</v>
       </c>
-      <c r="D28" t="s">
+      <c r="I28" t="s">
         <v>666</v>
-      </c>
-      <c r="E28" t="s">
-        <v>514</v>
-      </c>
-      <c r="F28" t="s">
-        <v>574</v>
-      </c>
-      <c r="G28" t="s">
-        <v>667</v>
-      </c>
-      <c r="H28" t="s">
-        <v>668</v>
-      </c>
-      <c r="I28" t="s">
-        <v>669</v>
       </c>
     </row>
     <row r="29" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B29" t="s">
-        <v>724</v>
+        <v>667</v>
       </c>
       <c r="C29" t="s">
+        <v>668</v>
+      </c>
+      <c r="D29" t="s">
+        <v>669</v>
+      </c>
+      <c r="E29" t="s">
+        <v>512</v>
+      </c>
+      <c r="F29" t="s">
+        <v>531</v>
+      </c>
+      <c r="G29" t="s">
+        <v>361</v>
+      </c>
+      <c r="H29" t="s">
+        <v>136</v>
+      </c>
+      <c r="I29" t="s">
         <v>670</v>
-      </c>
-      <c r="D29" t="s">
-        <v>671</v>
-      </c>
-      <c r="E29" t="s">
-        <v>514</v>
-      </c>
-      <c r="F29" t="s">
-        <v>529</v>
-      </c>
-      <c r="G29" t="s">
-        <v>672</v>
-      </c>
-      <c r="H29" t="s">
-        <v>673</v>
-      </c>
-      <c r="I29" t="s">
-        <v>674</v>
       </c>
     </row>
     <row r="30" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B30" t="s">
-        <v>675</v>
+        <v>671</v>
       </c>
       <c r="C30" t="s">
-        <v>676</v>
+        <v>672</v>
       </c>
       <c r="D30" t="s">
-        <v>677</v>
+        <v>673</v>
       </c>
       <c r="E30" t="s">
-        <v>514</v>
+        <v>13</v>
       </c>
       <c r="F30" t="s">
-        <v>533</v>
+        <v>162</v>
       </c>
       <c r="G30" t="s">
-        <v>361</v>
+        <v>22</v>
       </c>
       <c r="H30" t="s">
-        <v>136</v>
+        <v>23</v>
       </c>
       <c r="I30" t="s">
-        <v>678</v>
+        <v>674</v>
       </c>
     </row>
     <row r="31" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B31" t="s">
-        <v>679</v>
+        <v>675</v>
       </c>
       <c r="C31" t="s">
-        <v>680</v>
+        <v>676</v>
       </c>
       <c r="D31" t="s">
-        <v>681</v>
+        <v>677</v>
       </c>
       <c r="E31" t="s">
         <v>13</v>
       </c>
       <c r="F31" t="s">
-        <v>162</v>
+        <v>91</v>
       </c>
       <c r="G31" t="s">
-        <v>22</v>
+        <v>438</v>
       </c>
       <c r="H31" t="s">
-        <v>23</v>
+        <v>57</v>
       </c>
       <c r="I31" t="s">
-        <v>682</v>
+        <v>678</v>
       </c>
     </row>
     <row r="32" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B32" t="s">
-        <v>683</v>
+        <v>679</v>
       </c>
       <c r="C32" t="s">
-        <v>684</v>
+        <v>680</v>
       </c>
       <c r="D32" t="s">
-        <v>685</v>
+        <v>681</v>
       </c>
       <c r="E32" t="s">
         <v>13</v>
@@ -5961,195 +6058,221 @@
         <v>91</v>
       </c>
       <c r="G32" t="s">
-        <v>439</v>
+        <v>682</v>
       </c>
       <c r="H32" t="s">
-        <v>57</v>
+        <v>683</v>
       </c>
       <c r="I32" t="s">
-        <v>686</v>
+        <v>684</v>
       </c>
     </row>
     <row r="33" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B33" t="s">
+        <v>685</v>
+      </c>
+      <c r="C33" t="s">
+        <v>686</v>
+      </c>
+      <c r="D33" t="s">
         <v>687</v>
       </c>
-      <c r="C33" t="s">
+      <c r="E33" t="s">
+        <v>13</v>
+      </c>
+      <c r="F33" t="s">
+        <v>21</v>
+      </c>
+      <c r="G33" t="s">
         <v>688</v>
       </c>
-      <c r="D33" t="s">
+      <c r="H33" t="s">
         <v>689</v>
       </c>
-      <c r="E33" t="s">
-        <v>13</v>
-      </c>
-      <c r="F33" t="s">
-        <v>91</v>
-      </c>
-      <c r="G33" t="s">
+      <c r="I33" t="s">
         <v>690</v>
-      </c>
-      <c r="H33" t="s">
-        <v>691</v>
-      </c>
-      <c r="I33" t="s">
-        <v>692</v>
       </c>
     </row>
     <row r="34" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B34" t="s">
+        <v>691</v>
+      </c>
+      <c r="C34" t="s">
+        <v>692</v>
+      </c>
+      <c r="D34" t="s">
         <v>693</v>
       </c>
-      <c r="C34" t="s">
+      <c r="E34" t="s">
+        <v>13</v>
+      </c>
+      <c r="F34" t="s">
+        <v>14</v>
+      </c>
+      <c r="G34" t="s">
+        <v>336</v>
+      </c>
+      <c r="H34" t="s">
+        <v>337</v>
+      </c>
+      <c r="I34" t="s">
         <v>694</v>
-      </c>
-      <c r="D34" t="s">
-        <v>695</v>
-      </c>
-      <c r="E34" t="s">
-        <v>13</v>
-      </c>
-      <c r="F34" t="s">
-        <v>21</v>
-      </c>
-      <c r="G34" t="s">
-        <v>696</v>
-      </c>
-      <c r="H34" t="s">
-        <v>697</v>
-      </c>
-      <c r="I34" t="s">
-        <v>698</v>
       </c>
     </row>
     <row r="35" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B35" t="s">
-        <v>699</v>
+        <v>695</v>
       </c>
       <c r="C35" t="s">
-        <v>700</v>
+        <v>696</v>
       </c>
       <c r="D35" t="s">
-        <v>701</v>
+        <v>697</v>
       </c>
       <c r="E35" t="s">
         <v>13</v>
       </c>
       <c r="F35" t="s">
-        <v>14</v>
+        <v>91</v>
       </c>
       <c r="G35" t="s">
-        <v>336</v>
+        <v>56</v>
       </c>
       <c r="H35" t="s">
-        <v>337</v>
+        <v>57</v>
       </c>
       <c r="I35" t="s">
-        <v>702</v>
+        <v>698</v>
       </c>
     </row>
     <row r="36" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B36" t="s">
+        <v>714</v>
+      </c>
+      <c r="C36" t="s">
+        <v>699</v>
+      </c>
+      <c r="D36" t="s">
+        <v>700</v>
+      </c>
+      <c r="E36" t="s">
+        <v>512</v>
+      </c>
+      <c r="F36" t="s">
+        <v>572</v>
+      </c>
+      <c r="G36" t="s">
+        <v>701</v>
+      </c>
+      <c r="H36" t="s">
+        <v>702</v>
+      </c>
+      <c r="I36" t="s">
         <v>703</v>
-      </c>
-      <c r="C36" t="s">
-        <v>704</v>
-      </c>
-      <c r="D36" t="s">
-        <v>705</v>
-      </c>
-      <c r="E36" t="s">
-        <v>13</v>
-      </c>
-      <c r="F36" t="s">
-        <v>91</v>
-      </c>
-      <c r="G36" t="s">
-        <v>56</v>
-      </c>
-      <c r="H36" t="s">
-        <v>57</v>
-      </c>
-      <c r="I36" t="s">
-        <v>706</v>
       </c>
     </row>
     <row r="37" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B37" t="s">
-        <v>722</v>
+        <v>715</v>
       </c>
       <c r="C37" t="s">
-        <v>707</v>
+        <v>699</v>
       </c>
       <c r="D37" t="s">
-        <v>708</v>
+        <v>704</v>
       </c>
       <c r="E37" t="s">
-        <v>514</v>
+        <v>13</v>
       </c>
       <c r="F37" t="s">
-        <v>580</v>
+        <v>705</v>
       </c>
       <c r="G37" t="s">
-        <v>709</v>
+        <v>336</v>
       </c>
       <c r="H37" t="s">
-        <v>710</v>
+        <v>337</v>
       </c>
       <c r="I37" t="s">
-        <v>711</v>
+        <v>706</v>
       </c>
     </row>
     <row r="38" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B38" t="s">
-        <v>723</v>
+        <v>707</v>
       </c>
       <c r="C38" t="s">
-        <v>707</v>
+        <v>708</v>
       </c>
       <c r="D38" t="s">
-        <v>712</v>
+        <v>709</v>
       </c>
       <c r="E38" t="s">
-        <v>13</v>
+        <v>512</v>
       </c>
       <c r="F38" t="s">
-        <v>713</v>
+        <v>566</v>
       </c>
       <c r="G38" t="s">
-        <v>336</v>
+        <v>355</v>
       </c>
       <c r="H38" t="s">
         <v>337</v>
       </c>
       <c r="I38" t="s">
-        <v>714</v>
+        <v>710</v>
       </c>
     </row>
     <row r="39" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B39" t="s">
-        <v>715</v>
+        <v>729</v>
       </c>
       <c r="C39" t="s">
-        <v>716</v>
+        <v>730</v>
       </c>
       <c r="D39" t="s">
-        <v>717</v>
+        <v>731</v>
       </c>
       <c r="E39" t="s">
-        <v>514</v>
+        <v>736</v>
       </c>
       <c r="F39" t="s">
-        <v>574</v>
+        <v>91</v>
       </c>
       <c r="G39" t="s">
-        <v>355</v>
+        <v>732</v>
       </c>
       <c r="H39" t="s">
-        <v>337</v>
+        <v>733</v>
       </c>
       <c r="I39" t="s">
-        <v>718</v>
+        <v>734</v>
+      </c>
+    </row>
+    <row r="40" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B40" t="s">
+        <v>735</v>
+      </c>
+      <c r="C40" t="s">
+        <v>739</v>
+      </c>
+      <c r="D40" t="s">
+        <v>741</v>
+      </c>
+      <c r="E40" t="s">
+        <v>736</v>
+      </c>
+      <c r="F40" t="s">
+        <v>212</v>
+      </c>
+      <c r="G40" t="s">
+        <v>737</v>
+      </c>
+      <c r="H40" t="s">
+        <v>738</v>
+      </c>
+      <c r="I40" t="s">
+        <v>740</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Publish 20260813 REITs map update
</commit_message>
<xml_diff>
--- a/REITs_location_updating.xlsx
+++ b/REITs_location_updating.xlsx
@@ -8,15 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\21076\Desktop\公募REITs地图项目\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A36BD83A-DA40-485A-A807-F7E72CCA7C77}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EB2368FB-252D-4BA1-868F-9D49B41218A7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="已上市REITs" sheetId="1" r:id="rId1"/>
     <sheet name="未上市REITs" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="0" iterate="1" calcOnSave="0" concurrentManualCount="64"/>
+  <calcPr calcId="0" iterate="1" calcCompleted="0" calcOnSave="0" concurrentManualCount="64"/>
   <extLst>
     <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
       <xlwcv:version setVersion="1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1113" uniqueCount="742">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1114" uniqueCount="744">
   <si>
     <t>证券代码</t>
   </si>
@@ -1625,21 +1625,6 @@
   </si>
   <si>
     <t>{鼎保大厦，鼎博大厦}</t>
-  </si>
-  <si>
-    <t>华泰三峡清洁能源</t>
-  </si>
-  <si>
-    <t>中国三峡新能源（集团）股份有限公司</t>
-  </si>
-  <si>
-    <t>大连市庄河Ⅲ（300MW）海上风电场项目</t>
-  </si>
-  <si>
-    <t>大连市</t>
-  </si>
-  <si>
-    <t>{大连市庄河Ⅲ（300MW）海上风电场项目}</t>
   </si>
   <si>
     <t>博时山东铁投路桥</t>
@@ -2282,6 +2267,34 @@
   </si>
   <si>
     <t xml:space="preserve">A-7数据中心，A-8数据中心 </t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>华泰三峡清洁能源</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>508059.SH</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>中国三峡新能源（集团）股份有限公司</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>大连市庄河Ⅲ（300MW）海上风电场项目</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>大连市</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>辽宁省</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>{大连市庄河Ⅲ（300MW）海上风电场项目}</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
@@ -2649,10 +2662,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I88"/>
+  <dimension ref="A1:I89"/>
   <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="2" width="12" customWidth="1"/>
+    <col min="1" max="1" width="12" customWidth="1"/>
+    <col min="2" max="2" width="27.54296875" customWidth="1"/>
     <col min="3" max="4" width="48" customWidth="1"/>
     <col min="5" max="8" width="12" customWidth="1"/>
     <col min="9" max="9" width="48" customWidth="1"/>
@@ -4627,7 +4641,7 @@
         <v>424</v>
       </c>
       <c r="I68" t="s">
-        <v>726</v>
+        <v>721</v>
       </c>
     </row>
     <row r="69" spans="1:9" x14ac:dyDescent="0.25">
@@ -4693,7 +4707,7 @@
         <v>435</v>
       </c>
       <c r="B71" t="s">
-        <v>717</v>
+        <v>712</v>
       </c>
       <c r="C71" t="s">
         <v>436</v>
@@ -4972,7 +4986,7 @@
         <v>489</v>
       </c>
       <c r="H80" t="s">
-        <v>723</v>
+        <v>718</v>
       </c>
       <c r="I80" t="s">
         <v>490</v>
@@ -5059,7 +5073,7 @@
         <v>506</v>
       </c>
       <c r="H83" t="s">
-        <v>724</v>
+        <v>719</v>
       </c>
       <c r="I83" t="s">
         <v>507</v>
@@ -5154,7 +5168,7 @@
     </row>
     <row r="87" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
-        <v>711</v>
+        <v>706</v>
       </c>
       <c r="B87" t="s">
         <v>529</v>
@@ -5163,7 +5177,7 @@
         <v>530</v>
       </c>
       <c r="D87" t="s">
-        <v>712</v>
+        <v>707</v>
       </c>
       <c r="E87" t="s">
         <v>512</v>
@@ -5183,16 +5197,16 @@
     </row>
     <row r="88" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
-        <v>720</v>
+        <v>715</v>
       </c>
       <c r="B88" t="s">
-        <v>719</v>
+        <v>714</v>
       </c>
       <c r="C88" t="s">
-        <v>721</v>
+        <v>716</v>
       </c>
       <c r="D88" t="s">
-        <v>722</v>
+        <v>717</v>
       </c>
       <c r="E88" t="s">
         <v>13</v>
@@ -5201,13 +5215,42 @@
         <v>91</v>
       </c>
       <c r="G88" t="s">
-        <v>728</v>
+        <v>723</v>
       </c>
       <c r="H88" t="s">
-        <v>725</v>
+        <v>720</v>
       </c>
       <c r="I88" t="s">
-        <v>727</v>
+        <v>722</v>
+      </c>
+    </row>
+    <row r="89" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A89" t="s">
+        <v>738</v>
+      </c>
+      <c r="B89" t="s">
+        <v>737</v>
+      </c>
+      <c r="C89" t="s">
+        <v>739</v>
+      </c>
+      <c r="D89" t="s">
+        <v>740</v>
+      </c>
+      <c r="E89" t="s">
+        <v>13</v>
+      </c>
+      <c r="F89" t="s">
+        <v>91</v>
+      </c>
+      <c r="G89" t="s">
+        <v>741</v>
+      </c>
+      <c r="H89" t="s">
+        <v>742</v>
+      </c>
+      <c r="I89" t="s">
+        <v>743</v>
       </c>
     </row>
   </sheetData>
@@ -5218,7 +5261,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:I40"/>
+  <dimension ref="A1:I39"/>
   <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -5275,65 +5318,65 @@
         <v>13</v>
       </c>
       <c r="F2" t="s">
-        <v>91</v>
+        <v>21</v>
       </c>
       <c r="G2" t="s">
+        <v>273</v>
+      </c>
+      <c r="H2" t="s">
+        <v>57</v>
+      </c>
+      <c r="I2" t="s">
         <v>536</v>
-      </c>
-      <c r="H2" t="s">
-        <v>156</v>
-      </c>
-      <c r="I2" t="s">
-        <v>537</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="B3" t="s">
+        <v>537</v>
+      </c>
+      <c r="C3" t="s">
         <v>538</v>
       </c>
-      <c r="C3" t="s">
+      <c r="D3" t="s">
         <v>539</v>
       </c>
-      <c r="D3" t="s">
+      <c r="E3" t="s">
+        <v>13</v>
+      </c>
+      <c r="F3" t="s">
+        <v>272</v>
+      </c>
+      <c r="G3" t="s">
         <v>540</v>
       </c>
-      <c r="E3" t="s">
-        <v>13</v>
-      </c>
-      <c r="F3" t="s">
-        <v>21</v>
-      </c>
-      <c r="G3" t="s">
-        <v>273</v>
-      </c>
       <c r="H3" t="s">
-        <v>57</v>
+        <v>541</v>
       </c>
       <c r="I3" t="s">
-        <v>541</v>
+        <v>542</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="B4" t="s">
-        <v>542</v>
+        <v>543</v>
       </c>
       <c r="C4" t="s">
-        <v>543</v>
+        <v>544</v>
       </c>
       <c r="D4" t="s">
-        <v>544</v>
+        <v>545</v>
       </c>
       <c r="E4" t="s">
         <v>13</v>
       </c>
       <c r="F4" t="s">
-        <v>272</v>
+        <v>21</v>
       </c>
       <c r="G4" t="s">
-        <v>545</v>
+        <v>546</v>
       </c>
       <c r="H4" t="s">
-        <v>546</v>
+        <v>112</v>
       </c>
       <c r="I4" t="s">
         <v>547</v>
@@ -5353,27 +5396,27 @@
         <v>13</v>
       </c>
       <c r="F5" t="s">
-        <v>21</v>
+        <v>14</v>
       </c>
       <c r="G5" t="s">
+        <v>514</v>
+      </c>
+      <c r="H5" t="s">
+        <v>515</v>
+      </c>
+      <c r="I5" t="s">
         <v>551</v>
-      </c>
-      <c r="H5" t="s">
-        <v>112</v>
-      </c>
-      <c r="I5" t="s">
-        <v>552</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="B6" t="s">
+        <v>552</v>
+      </c>
+      <c r="C6" t="s">
         <v>553</v>
       </c>
-      <c r="C6" t="s">
+      <c r="D6" t="s">
         <v>554</v>
-      </c>
-      <c r="D6" t="s">
-        <v>555</v>
       </c>
       <c r="E6" t="s">
         <v>13</v>
@@ -5382,91 +5425,91 @@
         <v>14</v>
       </c>
       <c r="G6" t="s">
-        <v>514</v>
+        <v>205</v>
       </c>
       <c r="H6" t="s">
-        <v>515</v>
+        <v>206</v>
       </c>
       <c r="I6" t="s">
-        <v>556</v>
+        <v>555</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="B7" t="s">
+        <v>713</v>
+      </c>
+      <c r="C7" t="s">
+        <v>436</v>
+      </c>
+      <c r="D7" t="s">
+        <v>556</v>
+      </c>
+      <c r="E7" t="s">
+        <v>13</v>
+      </c>
+      <c r="F7" t="s">
+        <v>29</v>
+      </c>
+      <c r="G7" t="s">
+        <v>142</v>
+      </c>
+      <c r="H7" t="s">
+        <v>143</v>
+      </c>
+      <c r="I7" t="s">
         <v>557</v>
-      </c>
-      <c r="C7" t="s">
-        <v>558</v>
-      </c>
-      <c r="D7" t="s">
-        <v>559</v>
-      </c>
-      <c r="E7" t="s">
-        <v>13</v>
-      </c>
-      <c r="F7" t="s">
-        <v>14</v>
-      </c>
-      <c r="G7" t="s">
-        <v>205</v>
-      </c>
-      <c r="H7" t="s">
-        <v>206</v>
-      </c>
-      <c r="I7" t="s">
-        <v>560</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="B8" t="s">
-        <v>718</v>
+        <v>558</v>
       </c>
       <c r="C8" t="s">
-        <v>436</v>
+        <v>559</v>
       </c>
       <c r="D8" t="s">
+        <v>560</v>
+      </c>
+      <c r="E8" t="s">
+        <v>512</v>
+      </c>
+      <c r="F8" t="s">
         <v>561</v>
       </c>
-      <c r="E8" t="s">
-        <v>13</v>
-      </c>
-      <c r="F8" t="s">
-        <v>29</v>
-      </c>
       <c r="G8" t="s">
-        <v>142</v>
+        <v>562</v>
       </c>
       <c r="H8" t="s">
-        <v>143</v>
+        <v>563</v>
       </c>
       <c r="I8" t="s">
-        <v>562</v>
+        <v>708</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="B9" t="s">
-        <v>563</v>
+        <v>564</v>
       </c>
       <c r="C9" t="s">
-        <v>564</v>
+        <v>565</v>
       </c>
       <c r="D9" t="s">
-        <v>565</v>
+        <v>566</v>
       </c>
       <c r="E9" t="s">
         <v>512</v>
       </c>
       <c r="F9" t="s">
-        <v>566</v>
+        <v>567</v>
       </c>
       <c r="G9" t="s">
-        <v>567</v>
+        <v>15</v>
       </c>
       <c r="H9" t="s">
+        <v>15</v>
+      </c>
+      <c r="I9" t="s">
         <v>568</v>
-      </c>
-      <c r="I9" t="s">
-        <v>713</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.25">
@@ -5486,62 +5529,62 @@
         <v>572</v>
       </c>
       <c r="G10" t="s">
-        <v>15</v>
+        <v>573</v>
       </c>
       <c r="H10" t="s">
-        <v>15</v>
+        <v>574</v>
       </c>
       <c r="I10" t="s">
-        <v>573</v>
+        <v>575</v>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="B11" t="s">
-        <v>574</v>
+        <v>576</v>
       </c>
       <c r="C11" t="s">
-        <v>575</v>
+        <v>577</v>
       </c>
       <c r="D11" t="s">
-        <v>576</v>
+        <v>578</v>
       </c>
       <c r="E11" t="s">
         <v>512</v>
       </c>
       <c r="F11" t="s">
-        <v>577</v>
+        <v>527</v>
       </c>
       <c r="G11" t="s">
-        <v>578</v>
+        <v>343</v>
       </c>
       <c r="H11" t="s">
+        <v>344</v>
+      </c>
+      <c r="I11" t="s">
         <v>579</v>
-      </c>
-      <c r="I11" t="s">
-        <v>580</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="B12" t="s">
+        <v>580</v>
+      </c>
+      <c r="C12" t="s">
         <v>581</v>
       </c>
-      <c r="C12" t="s">
+      <c r="D12" t="s">
         <v>582</v>
-      </c>
-      <c r="D12" t="s">
-        <v>583</v>
       </c>
       <c r="E12" t="s">
         <v>512</v>
       </c>
       <c r="F12" t="s">
-        <v>527</v>
+        <v>567</v>
       </c>
       <c r="G12" t="s">
-        <v>343</v>
+        <v>583</v>
       </c>
       <c r="H12" t="s">
-        <v>344</v>
+        <v>412</v>
       </c>
       <c r="I12" t="s">
         <v>584</v>
@@ -5561,53 +5604,53 @@
         <v>512</v>
       </c>
       <c r="F13" t="s">
-        <v>572</v>
+        <v>561</v>
       </c>
       <c r="G13" t="s">
         <v>588</v>
       </c>
       <c r="H13" t="s">
-        <v>412</v>
+        <v>589</v>
       </c>
       <c r="I13" t="s">
-        <v>589</v>
+        <v>590</v>
       </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.25">
       <c r="B14" t="s">
-        <v>590</v>
+        <v>591</v>
       </c>
       <c r="C14" t="s">
-        <v>591</v>
+        <v>592</v>
       </c>
       <c r="D14" t="s">
-        <v>592</v>
+        <v>593</v>
       </c>
       <c r="E14" t="s">
         <v>512</v>
       </c>
       <c r="F14" t="s">
-        <v>566</v>
+        <v>527</v>
       </c>
       <c r="G14" t="s">
-        <v>593</v>
+        <v>594</v>
       </c>
       <c r="H14" t="s">
-        <v>594</v>
+        <v>595</v>
       </c>
       <c r="I14" t="s">
-        <v>595</v>
+        <v>596</v>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.25">
       <c r="B15" t="s">
-        <v>596</v>
+        <v>597</v>
       </c>
       <c r="C15" t="s">
-        <v>597</v>
+        <v>598</v>
       </c>
       <c r="D15" t="s">
-        <v>598</v>
+        <v>599</v>
       </c>
       <c r="E15" t="s">
         <v>512</v>
@@ -5616,36 +5659,36 @@
         <v>527</v>
       </c>
       <c r="G15" t="s">
-        <v>599</v>
+        <v>15</v>
       </c>
       <c r="H15" t="s">
+        <v>15</v>
+      </c>
+      <c r="I15" t="s">
         <v>600</v>
-      </c>
-      <c r="I15" t="s">
-        <v>601</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.25">
       <c r="B16" t="s">
+        <v>601</v>
+      </c>
+      <c r="C16" t="s">
         <v>602</v>
       </c>
-      <c r="C16" t="s">
+      <c r="D16" t="s">
         <v>603</v>
       </c>
-      <c r="D16" t="s">
+      <c r="E16" t="s">
+        <v>13</v>
+      </c>
+      <c r="F16" t="s">
         <v>604</v>
       </c>
-      <c r="E16" t="s">
-        <v>512</v>
-      </c>
-      <c r="F16" t="s">
-        <v>527</v>
-      </c>
       <c r="G16" t="s">
-        <v>15</v>
+        <v>129</v>
       </c>
       <c r="H16" t="s">
-        <v>15</v>
+        <v>129</v>
       </c>
       <c r="I16" t="s">
         <v>605</v>
@@ -5665,53 +5708,53 @@
         <v>13</v>
       </c>
       <c r="F17" t="s">
+        <v>91</v>
+      </c>
+      <c r="G17" t="s">
         <v>609</v>
       </c>
-      <c r="G17" t="s">
-        <v>129</v>
-      </c>
       <c r="H17" t="s">
-        <v>129</v>
+        <v>610</v>
       </c>
       <c r="I17" t="s">
-        <v>610</v>
+        <v>611</v>
       </c>
     </row>
     <row r="18" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B18" t="s">
-        <v>611</v>
+        <v>612</v>
       </c>
       <c r="C18" t="s">
-        <v>612</v>
+        <v>613</v>
       </c>
       <c r="D18" t="s">
-        <v>613</v>
+        <v>614</v>
       </c>
       <c r="E18" t="s">
-        <v>13</v>
+        <v>512</v>
       </c>
       <c r="F18" t="s">
-        <v>91</v>
+        <v>527</v>
       </c>
       <c r="G18" t="s">
-        <v>614</v>
+        <v>35</v>
       </c>
       <c r="H18" t="s">
+        <v>35</v>
+      </c>
+      <c r="I18" t="s">
         <v>615</v>
-      </c>
-      <c r="I18" t="s">
-        <v>616</v>
       </c>
     </row>
     <row r="19" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B19" t="s">
+        <v>616</v>
+      </c>
+      <c r="C19" t="s">
         <v>617</v>
       </c>
-      <c r="C19" t="s">
+      <c r="D19" t="s">
         <v>618</v>
-      </c>
-      <c r="D19" t="s">
-        <v>619</v>
       </c>
       <c r="E19" t="s">
         <v>512</v>
@@ -5720,24 +5763,24 @@
         <v>527</v>
       </c>
       <c r="G19" t="s">
-        <v>35</v>
+        <v>619</v>
       </c>
       <c r="H19" t="s">
-        <v>35</v>
+        <v>620</v>
       </c>
       <c r="I19" t="s">
-        <v>620</v>
+        <v>621</v>
       </c>
     </row>
     <row r="20" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B20" t="s">
-        <v>621</v>
+        <v>622</v>
       </c>
       <c r="C20" t="s">
-        <v>622</v>
+        <v>623</v>
       </c>
       <c r="D20" t="s">
-        <v>623</v>
+        <v>624</v>
       </c>
       <c r="E20" t="s">
         <v>512</v>
@@ -5746,114 +5789,114 @@
         <v>527</v>
       </c>
       <c r="G20" t="s">
-        <v>624</v>
+        <v>336</v>
       </c>
       <c r="H20" t="s">
+        <v>337</v>
+      </c>
+      <c r="I20" t="s">
         <v>625</v>
-      </c>
-      <c r="I20" t="s">
-        <v>626</v>
       </c>
     </row>
     <row r="21" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B21" t="s">
+        <v>626</v>
+      </c>
+      <c r="C21" t="s">
         <v>627</v>
       </c>
-      <c r="C21" t="s">
+      <c r="D21" t="s">
         <v>628</v>
-      </c>
-      <c r="D21" t="s">
-        <v>629</v>
       </c>
       <c r="E21" t="s">
         <v>512</v>
       </c>
       <c r="F21" t="s">
-        <v>527</v>
+        <v>629</v>
       </c>
       <c r="G21" t="s">
-        <v>336</v>
+        <v>630</v>
       </c>
       <c r="H21" t="s">
-        <v>337</v>
+        <v>631</v>
       </c>
       <c r="I21" t="s">
-        <v>630</v>
+        <v>632</v>
       </c>
     </row>
     <row r="22" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B22" t="s">
-        <v>631</v>
+        <v>633</v>
       </c>
       <c r="C22" t="s">
-        <v>632</v>
+        <v>634</v>
       </c>
       <c r="D22" t="s">
-        <v>633</v>
+        <v>635</v>
       </c>
       <c r="E22" t="s">
         <v>512</v>
       </c>
       <c r="F22" t="s">
-        <v>634</v>
+        <v>567</v>
       </c>
       <c r="G22" t="s">
-        <v>635</v>
+        <v>35</v>
       </c>
       <c r="H22" t="s">
+        <v>35</v>
+      </c>
+      <c r="I22" t="s">
         <v>636</v>
-      </c>
-      <c r="I22" t="s">
-        <v>637</v>
       </c>
     </row>
     <row r="23" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B23" t="s">
+        <v>637</v>
+      </c>
+      <c r="C23" t="s">
         <v>638</v>
       </c>
-      <c r="C23" t="s">
+      <c r="D23" t="s">
         <v>639</v>
       </c>
-      <c r="D23" t="s">
+      <c r="E23" t="s">
+        <v>13</v>
+      </c>
+      <c r="F23" t="s">
+        <v>162</v>
+      </c>
+      <c r="G23" t="s">
+        <v>15</v>
+      </c>
+      <c r="H23" t="s">
+        <v>15</v>
+      </c>
+      <c r="I23" t="s">
         <v>640</v>
-      </c>
-      <c r="E23" t="s">
-        <v>512</v>
-      </c>
-      <c r="F23" t="s">
-        <v>572</v>
-      </c>
-      <c r="G23" t="s">
-        <v>35</v>
-      </c>
-      <c r="H23" t="s">
-        <v>35</v>
-      </c>
-      <c r="I23" t="s">
-        <v>641</v>
       </c>
     </row>
     <row r="24" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B24" t="s">
+        <v>641</v>
+      </c>
+      <c r="C24" t="s">
         <v>642</v>
       </c>
-      <c r="C24" t="s">
+      <c r="D24" t="s">
         <v>643</v>
       </c>
-      <c r="D24" t="s">
+      <c r="E24" t="s">
+        <v>13</v>
+      </c>
+      <c r="F24" t="s">
+        <v>471</v>
+      </c>
+      <c r="G24" t="s">
         <v>644</v>
       </c>
-      <c r="E24" t="s">
-        <v>13</v>
-      </c>
-      <c r="F24" t="s">
-        <v>162</v>
-      </c>
-      <c r="G24" t="s">
-        <v>15</v>
-      </c>
       <c r="H24" t="s">
-        <v>15</v>
+        <v>412</v>
       </c>
       <c r="I24" t="s">
         <v>645</v>
@@ -5873,13 +5916,13 @@
         <v>13</v>
       </c>
       <c r="F25" t="s">
-        <v>471</v>
+        <v>187</v>
       </c>
       <c r="G25" t="s">
         <v>649</v>
       </c>
       <c r="H25" t="s">
-        <v>412</v>
+        <v>23</v>
       </c>
       <c r="I25" t="s">
         <v>650</v>
@@ -5896,24 +5939,24 @@
         <v>653</v>
       </c>
       <c r="E26" t="s">
-        <v>13</v>
+        <v>512</v>
       </c>
       <c r="F26" t="s">
-        <v>187</v>
+        <v>561</v>
       </c>
       <c r="G26" t="s">
         <v>654</v>
       </c>
       <c r="H26" t="s">
-        <v>23</v>
+        <v>655</v>
       </c>
       <c r="I26" t="s">
-        <v>655</v>
+        <v>656</v>
       </c>
     </row>
     <row r="27" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B27" t="s">
-        <v>656</v>
+        <v>711</v>
       </c>
       <c r="C27" t="s">
         <v>657</v>
@@ -5925,7 +5968,7 @@
         <v>512</v>
       </c>
       <c r="F27" t="s">
-        <v>566</v>
+        <v>527</v>
       </c>
       <c r="G27" t="s">
         <v>659</v>
@@ -5939,91 +5982,91 @@
     </row>
     <row r="28" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B28" t="s">
-        <v>716</v>
+        <v>662</v>
       </c>
       <c r="C28" t="s">
-        <v>662</v>
+        <v>663</v>
       </c>
       <c r="D28" t="s">
-        <v>663</v>
+        <v>664</v>
       </c>
       <c r="E28" t="s">
         <v>512</v>
       </c>
       <c r="F28" t="s">
-        <v>527</v>
+        <v>531</v>
       </c>
       <c r="G28" t="s">
-        <v>664</v>
+        <v>361</v>
       </c>
       <c r="H28" t="s">
+        <v>136</v>
+      </c>
+      <c r="I28" t="s">
         <v>665</v>
-      </c>
-      <c r="I28" t="s">
-        <v>666</v>
       </c>
     </row>
     <row r="29" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B29" t="s">
+        <v>666</v>
+      </c>
+      <c r="C29" t="s">
         <v>667</v>
       </c>
-      <c r="C29" t="s">
+      <c r="D29" t="s">
         <v>668</v>
       </c>
-      <c r="D29" t="s">
+      <c r="E29" t="s">
+        <v>13</v>
+      </c>
+      <c r="F29" t="s">
+        <v>162</v>
+      </c>
+      <c r="G29" t="s">
+        <v>22</v>
+      </c>
+      <c r="H29" t="s">
+        <v>23</v>
+      </c>
+      <c r="I29" t="s">
         <v>669</v>
-      </c>
-      <c r="E29" t="s">
-        <v>512</v>
-      </c>
-      <c r="F29" t="s">
-        <v>531</v>
-      </c>
-      <c r="G29" t="s">
-        <v>361</v>
-      </c>
-      <c r="H29" t="s">
-        <v>136</v>
-      </c>
-      <c r="I29" t="s">
-        <v>670</v>
       </c>
     </row>
     <row r="30" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B30" t="s">
+        <v>670</v>
+      </c>
+      <c r="C30" t="s">
         <v>671</v>
       </c>
-      <c r="C30" t="s">
+      <c r="D30" t="s">
         <v>672</v>
       </c>
-      <c r="D30" t="s">
+      <c r="E30" t="s">
+        <v>13</v>
+      </c>
+      <c r="F30" t="s">
+        <v>91</v>
+      </c>
+      <c r="G30" t="s">
+        <v>438</v>
+      </c>
+      <c r="H30" t="s">
+        <v>57</v>
+      </c>
+      <c r="I30" t="s">
         <v>673</v>
-      </c>
-      <c r="E30" t="s">
-        <v>13</v>
-      </c>
-      <c r="F30" t="s">
-        <v>162</v>
-      </c>
-      <c r="G30" t="s">
-        <v>22</v>
-      </c>
-      <c r="H30" t="s">
-        <v>23</v>
-      </c>
-      <c r="I30" t="s">
-        <v>674</v>
       </c>
     </row>
     <row r="31" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B31" t="s">
+        <v>674</v>
+      </c>
+      <c r="C31" t="s">
         <v>675</v>
       </c>
-      <c r="C31" t="s">
+      <c r="D31" t="s">
         <v>676</v>
-      </c>
-      <c r="D31" t="s">
-        <v>677</v>
       </c>
       <c r="E31" t="s">
         <v>13</v>
@@ -6032,114 +6075,114 @@
         <v>91</v>
       </c>
       <c r="G31" t="s">
-        <v>438</v>
+        <v>677</v>
       </c>
       <c r="H31" t="s">
-        <v>57</v>
+        <v>678</v>
       </c>
       <c r="I31" t="s">
-        <v>678</v>
+        <v>679</v>
       </c>
     </row>
     <row r="32" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B32" t="s">
-        <v>679</v>
+        <v>680</v>
       </c>
       <c r="C32" t="s">
-        <v>680</v>
+        <v>681</v>
       </c>
       <c r="D32" t="s">
-        <v>681</v>
+        <v>682</v>
       </c>
       <c r="E32" t="s">
         <v>13</v>
       </c>
       <c r="F32" t="s">
-        <v>91</v>
+        <v>21</v>
       </c>
       <c r="G32" t="s">
-        <v>682</v>
+        <v>683</v>
       </c>
       <c r="H32" t="s">
-        <v>683</v>
+        <v>684</v>
       </c>
       <c r="I32" t="s">
-        <v>684</v>
+        <v>685</v>
       </c>
     </row>
     <row r="33" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B33" t="s">
-        <v>685</v>
+        <v>686</v>
       </c>
       <c r="C33" t="s">
-        <v>686</v>
+        <v>687</v>
       </c>
       <c r="D33" t="s">
-        <v>687</v>
+        <v>688</v>
       </c>
       <c r="E33" t="s">
         <v>13</v>
       </c>
       <c r="F33" t="s">
-        <v>21</v>
+        <v>14</v>
       </c>
       <c r="G33" t="s">
-        <v>688</v>
+        <v>336</v>
       </c>
       <c r="H33" t="s">
+        <v>337</v>
+      </c>
+      <c r="I33" t="s">
         <v>689</v>
-      </c>
-      <c r="I33" t="s">
-        <v>690</v>
       </c>
     </row>
     <row r="34" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B34" t="s">
+        <v>690</v>
+      </c>
+      <c r="C34" t="s">
         <v>691</v>
       </c>
-      <c r="C34" t="s">
+      <c r="D34" t="s">
         <v>692</v>
       </c>
-      <c r="D34" t="s">
+      <c r="E34" t="s">
+        <v>13</v>
+      </c>
+      <c r="F34" t="s">
+        <v>91</v>
+      </c>
+      <c r="G34" t="s">
+        <v>56</v>
+      </c>
+      <c r="H34" t="s">
+        <v>57</v>
+      </c>
+      <c r="I34" t="s">
         <v>693</v>
-      </c>
-      <c r="E34" t="s">
-        <v>13</v>
-      </c>
-      <c r="F34" t="s">
-        <v>14</v>
-      </c>
-      <c r="G34" t="s">
-        <v>336</v>
-      </c>
-      <c r="H34" t="s">
-        <v>337</v>
-      </c>
-      <c r="I34" t="s">
-        <v>694</v>
       </c>
     </row>
     <row r="35" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B35" t="s">
+        <v>709</v>
+      </c>
+      <c r="C35" t="s">
+        <v>694</v>
+      </c>
+      <c r="D35" t="s">
         <v>695</v>
       </c>
-      <c r="C35" t="s">
+      <c r="E35" t="s">
+        <v>512</v>
+      </c>
+      <c r="F35" t="s">
+        <v>567</v>
+      </c>
+      <c r="G35" t="s">
         <v>696</v>
       </c>
-      <c r="D35" t="s">
+      <c r="H35" t="s">
         <v>697</v>
-      </c>
-      <c r="E35" t="s">
-        <v>13</v>
-      </c>
-      <c r="F35" t="s">
-        <v>91</v>
-      </c>
-      <c r="G35" t="s">
-        <v>56</v>
-      </c>
-      <c r="H35" t="s">
-        <v>57</v>
       </c>
       <c r="I35" t="s">
         <v>698</v>
@@ -6147,97 +6190,97 @@
     </row>
     <row r="36" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B36" t="s">
-        <v>714</v>
+        <v>710</v>
       </c>
       <c r="C36" t="s">
+        <v>694</v>
+      </c>
+      <c r="D36" t="s">
         <v>699</v>
       </c>
-      <c r="D36" t="s">
+      <c r="E36" t="s">
+        <v>13</v>
+      </c>
+      <c r="F36" t="s">
         <v>700</v>
       </c>
-      <c r="E36" t="s">
-        <v>512</v>
-      </c>
-      <c r="F36" t="s">
-        <v>572</v>
-      </c>
       <c r="G36" t="s">
+        <v>336</v>
+      </c>
+      <c r="H36" t="s">
+        <v>337</v>
+      </c>
+      <c r="I36" t="s">
         <v>701</v>
-      </c>
-      <c r="H36" t="s">
-        <v>702</v>
-      </c>
-      <c r="I36" t="s">
-        <v>703</v>
       </c>
     </row>
     <row r="37" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B37" t="s">
-        <v>715</v>
+        <v>702</v>
       </c>
       <c r="C37" t="s">
-        <v>699</v>
+        <v>703</v>
       </c>
       <c r="D37" t="s">
         <v>704</v>
       </c>
       <c r="E37" t="s">
-        <v>13</v>
+        <v>512</v>
       </c>
       <c r="F37" t="s">
-        <v>705</v>
+        <v>561</v>
       </c>
       <c r="G37" t="s">
-        <v>336</v>
+        <v>355</v>
       </c>
       <c r="H37" t="s">
         <v>337</v>
       </c>
       <c r="I37" t="s">
-        <v>706</v>
+        <v>705</v>
       </c>
     </row>
     <row r="38" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B38" t="s">
-        <v>707</v>
+        <v>724</v>
       </c>
       <c r="C38" t="s">
-        <v>708</v>
+        <v>725</v>
       </c>
       <c r="D38" t="s">
-        <v>709</v>
+        <v>726</v>
       </c>
       <c r="E38" t="s">
-        <v>512</v>
+        <v>731</v>
       </c>
       <c r="F38" t="s">
-        <v>566</v>
+        <v>91</v>
       </c>
       <c r="G38" t="s">
-        <v>355</v>
+        <v>727</v>
       </c>
       <c r="H38" t="s">
-        <v>337</v>
+        <v>728</v>
       </c>
       <c r="I38" t="s">
-        <v>710</v>
+        <v>729</v>
       </c>
     </row>
     <row r="39" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B39" t="s">
-        <v>729</v>
+        <v>730</v>
       </c>
       <c r="C39" t="s">
-        <v>730</v>
+        <v>734</v>
       </c>
       <c r="D39" t="s">
+        <v>736</v>
+      </c>
+      <c r="E39" t="s">
         <v>731</v>
       </c>
-      <c r="E39" t="s">
-        <v>736</v>
-      </c>
       <c r="F39" t="s">
-        <v>91</v>
+        <v>212</v>
       </c>
       <c r="G39" t="s">
         <v>732</v>
@@ -6246,33 +6289,7 @@
         <v>733</v>
       </c>
       <c r="I39" t="s">
-        <v>734</v>
-      </c>
-    </row>
-    <row r="40" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B40" t="s">
         <v>735</v>
-      </c>
-      <c r="C40" t="s">
-        <v>739</v>
-      </c>
-      <c r="D40" t="s">
-        <v>741</v>
-      </c>
-      <c r="E40" t="s">
-        <v>736</v>
-      </c>
-      <c r="F40" t="s">
-        <v>212</v>
-      </c>
-      <c r="G40" t="s">
-        <v>737</v>
-      </c>
-      <c r="H40" t="s">
-        <v>738</v>
-      </c>
-      <c r="I40" t="s">
-        <v>740</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Apply confirmed REIT categories and relocate map template
</commit_message>
<xml_diff>
--- a/REITs_location_updating.xlsx
+++ b/REITs_location_updating.xlsx
@@ -6883,7 +6883,7 @@
       </c>
       <c r="F90" t="inlineStr">
         <is>
-          <t xml:space="preserve">办公+商业零售</t>
+          <t xml:space="preserve">办公</t>
         </is>
       </c>
       <c r="G90" t="inlineStr">
@@ -7296,7 +7296,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t xml:space="preserve">商业综合体</t>
+          <t xml:space="preserve">办公+商业零售</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -8543,7 +8543,7 @@
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t xml:space="preserve">购物中心</t>
+          <t xml:space="preserve">商业零售</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
@@ -8586,7 +8586,7 @@
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t xml:space="preserve">奥特莱斯+购物中心</t>
+          <t xml:space="preserve">奥特莱斯+商业零售</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
@@ -8629,7 +8629,7 @@
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t xml:space="preserve">购物中心</t>
+          <t xml:space="preserve">商业零售</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
@@ -8801,7 +8801,7 @@
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t xml:space="preserve">商业综合体+酒店</t>
+          <t xml:space="preserve">酒店+商业零售</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">

</xml_diff>